<commit_message>
New 6-day training split, injury-resilience/league-day rules, expanded agility exercise pool
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O254"/>
+  <dimension ref="A1:O261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15618,6 +15618,415 @@
       <c r="M254" s="9" t="inlineStr"/>
       <c r="N254" s="9" t="inlineStr"/>
       <c r="O254" s="9" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>CD-006</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Reactive Mirror Drill (Partner Shadow)</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Read-and-react change of direction — mirrors a partner's lateral/forward-back movement, closer to defending or getting open off a live cutter than a pre-planned cone pattern</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Stay on the balls of your feet and react to your partner's hips, not their eyes or the disc — mirror the movement a half-beat after it starts.</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>CD-005</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>CD-009</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>CD-007</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Curved Cut (Banana Route)</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>The rounded, decelerate-and-bend cutting mechanic used on deep/around cuts in ultimate, as opposed to a sharp planted cut</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Cones</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Requires Running Room (15-20 yd)</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Round the turn instead of planting hard — bend the path like a banana, leaning in and gradually opening back upfield rather than stopping and redirecting.</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>CD-003</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>CD-008</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Close-Space Juke / Hip Turn Drill</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>A tight-radius fake-and-go move trained in a small footprint — built for apartment/minimal-space athletes who can't get outside for full cone work</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Sell the fake with a real weight shift, then snap the hips and drive hard the other way — small space, but full-intent redirection.</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>CD-005</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>CD-007</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>CD-009</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Backpedal-to-Sprint Transition</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Defensive backpedal opening into a sprint — the mark/defender's transition from a defensive shuffle into a recovery sprint</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Requires Running Room (10 yd)</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Stay low in the backpedal, then snap the hips and drive forward the instant you flip — the transition should be one motion, not two.</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>CD-005</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>CD-006</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>CD-010</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>T-Drill (4-Direction Cone Drill)</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>A structured forward-shuffle-backpedal combination drill that layers all four directional change patterns in one rep</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Cones</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Requires Running Room (10-15 yd)</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Sprint the top, shuffle the crossbar, backpedal the stem — keep the hips low and the steps choppy through every direction change.</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>CD-004</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>CD-002</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>CD-011</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Single-Cone Reactive Cut (Visual Cue)</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>A coach- or partner-cued reactive cut off a visual signal — the closest cone-drill approximation of reading a defender and cutting on a break</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Cones or Partner</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Requires Running Room (Short)</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Wait for the cue before you commit — a late, sharp cut beats an early, telegraphed one every time.</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>CD-003</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>CD-006</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>CD-012</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Shuffle-to-Close-Out</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>The mark's close-out mechanic — a shuffle or sprint approach that decelerates under control into a balanced defensive stance</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Requires Running Room (5-10 yd)</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Close the distance under control and chop your steps down as you arrive — you want to land balanced and ready to move, not lunging in off-balance.</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>CD-005</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>CD-009</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O254"/>

</xml_diff>

<commit_message>
Add 19 new exercises; reconcile day-structure-templates.md with coach's corrected session order
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O261"/>
+  <dimension ref="A1:O286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13073,7 +13073,7 @@
       </c>
       <c r="E214" s="7" t="inlineStr">
         <is>
-          <t>Anti-extension core control with an added overhead plate-pass challenge; progression from the basic Dead Bug</t>
+          <t>Advanced anti-extension core control with an added overhead plate-pass challenge; the advanced-tier crunch-variation option alongside Weighted Sit-Up (CR-034)</t>
         </is>
       </c>
       <c r="F214" s="7" t="inlineStr">
@@ -13099,7 +13099,7 @@
       <c r="J214" s="7" t="inlineStr"/>
       <c r="K214" s="7" t="inlineStr">
         <is>
-          <t>Novice</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="L214" s="7" t="inlineStr">
@@ -16025,6 +16025,1683 @@
       <c r="L261" t="inlineStr">
         <is>
           <t>Year-round</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="7" t="inlineStr">
+        <is>
+          <t>RS-001</t>
+        </is>
+      </c>
+      <c r="B262" s="7" t="inlineStr">
+        <is>
+          <t>DB Loaded Lateral Bound (Entry)</t>
+        </is>
+      </c>
+      <c r="C262" s="7" t="inlineStr">
+        <is>
+          <t>Core 50</t>
+        </is>
+      </c>
+      <c r="D262" s="7" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E262" s="7" t="inlineStr">
+        <is>
+          <t>Entry point into a loaded, scaffolded progression that trains the separation cut (push off one leg, load and stick on the other) under external resistance rather than bodyweight alone — a distinct quality from unloaded plyometrics/reactive strength above</t>
+        </is>
+      </c>
+      <c r="F262" s="7" t="inlineStr">
+        <is>
+          <t>Light Dumbbells</t>
+        </is>
+      </c>
+      <c r="G262" s="7" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H262" s="7" t="inlineStr">
+        <is>
+          <t>Hold the dumbbells at your sides, push off one leg, and stick the landing dead still on the other before you reset — this is about control under load, not distance yet.</t>
+        </is>
+      </c>
+      <c r="I262" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J262" s="7" t="inlineStr">
+        <is>
+          <t>RS-002</t>
+        </is>
+      </c>
+      <c r="K262" s="7" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L262" s="7" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M262" s="7" t="n"/>
+      <c r="N262" s="7" t="n"/>
+      <c r="O262" s="7" t="inlineStr">
+        <is>
+          <t>New Reflexive Strength category (added when incorporating Garage Strength-style program design) — loaded, low-rep, scaffolded sport-movement-pattern work, distinct from the Plyometric/Jump (Reactive Strength) category above. This progression is our own build for ultimate's cutting/separation pattern, not a reused example from any outside source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>RS-002</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>DB Loaded Lateral Bound to Vertical Stick</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>Adds a change-of-plane finish (lateral load into a vertical stick) to the separation-cut pattern — middle link in the scaffolded progression, more complex than the entry bound but not yet the full expression</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Light-Moderate Dumbbells</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>Bound laterally like before, but this time finish by driving straight up into a stick — redirect the momentum from sideways to vertical without losing your landing control.</t>
+        </is>
+      </c>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>RS-001</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>RS-003</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L263" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M263" s="2" t="n"/>
+      <c r="N263" s="2" t="n"/>
+      <c r="O263" s="2" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>RS-003</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL to Loaded Lateral Bound (Full Expression)</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>Full expression of the separation-cut chain — a loaded single-leg hip-hinge load-up immediately converted into a maximal lateral bound, mirroring the load-and-explode mechanics of cutting away from a mark at full speed</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Moderate Dumbbells</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (Short)</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>Load into the single-leg RDL like you're settling into the cut, then explode sideways the instant you feel the stretch — the hinge and the bound should feel like one continuous motion, not two separate reps.</t>
+        </is>
+      </c>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>RS-002</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L264" s="2" t="inlineStr">
+        <is>
+          <t>Off-season</t>
+        </is>
+      </c>
+      <c r="M264" s="2" t="n"/>
+      <c r="N264" s="2" t="n"/>
+      <c r="O264" s="2" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="7" t="inlineStr">
+        <is>
+          <t>RS-004</t>
+        </is>
+      </c>
+      <c r="B265" s="7" t="inlineStr">
+        <is>
+          <t>KB Loaded Deceleration Step (Entry)</t>
+        </is>
+      </c>
+      <c r="C265" s="7" t="inlineStr">
+        <is>
+          <t>Core 50</t>
+        </is>
+      </c>
+      <c r="D265" s="7" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E265" s="7" t="inlineStr">
+        <is>
+          <t>Entry point into a second scaffolded chain training the mark/close-out pattern — a loaded deceleration into a held athletic stance, building the braking strength that underlies closing out on a thrower under control</t>
+        </is>
+      </c>
+      <c r="F265" s="7" t="inlineStr">
+        <is>
+          <t>Kettlebell</t>
+        </is>
+      </c>
+      <c r="G265" s="7" t="inlineStr">
+        <is>
+          <t>Requires Running Room (Short)</t>
+        </is>
+      </c>
+      <c r="H265" s="7" t="inlineStr">
+        <is>
+          <t>Hold the kettlebell at your chest, take two building steps, then plant hard and stick a low, balanced stance — the goal is stopping on a dime, not drifting through the landing.</t>
+        </is>
+      </c>
+      <c r="I265" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J265" s="7" t="inlineStr">
+        <is>
+          <t>RS-005</t>
+        </is>
+      </c>
+      <c r="K265" s="7" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L265" s="7" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M265" s="7" t="n"/>
+      <c r="N265" s="7" t="n"/>
+      <c r="O265" s="7" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>RS-005</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>KB Loaded Deceleration Step to Reactive Redirect</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>Adds a reactive re-acceleration off the decelerated stance — middle link in the mark/close-out chain, training the stop-and-go quality of staying attached to a cutter after closing the gap</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Kettlebell</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (Short)</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>Stick the deceleration exactly like before, but the second you're balanced, redirect and accelerate hard in a new direction on a coach or partner's call — the stick and the re-accel are one skill, not two.</t>
+        </is>
+      </c>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>RS-004</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>RS-006</t>
+        </is>
+      </c>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L266" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season, In-season</t>
+        </is>
+      </c>
+      <c r="M266" s="2" t="n"/>
+      <c r="N266" s="2" t="n"/>
+      <c r="O266" s="2" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>RS-006</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Loaded Single-Arm Deceleration to Overhead Reach</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>Full expression of the mark/close-out chain — a loaded, asymmetric deceleration finished with a reach overhead, mirroring the moment a defender closes out and contests a throw or a catch at full extension</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>Single Dumbbell</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (Short)</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>Decelerate off the outside foot with the dumbbell held to one side, stick it, and drive the free arm straight overhead like you're contesting a throw — stay balanced through the reach, don't just fall into it.</t>
+        </is>
+      </c>
+      <c r="I267" s="2" t="inlineStr">
+        <is>
+          <t>RS-005</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L267" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season, In-season</t>
+        </is>
+      </c>
+      <c r="M267" s="2" t="n"/>
+      <c r="N267" s="2" t="n"/>
+      <c r="O267" s="2" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="7" t="inlineStr">
+        <is>
+          <t>PJ-028</t>
+        </is>
+      </c>
+      <c r="B268" s="7" t="inlineStr">
+        <is>
+          <t>DB Jump</t>
+        </is>
+      </c>
+      <c r="C268" s="7" t="inlineStr">
+        <is>
+          <t>Core 50</t>
+        </is>
+      </c>
+      <c r="D268" s="7" t="inlineStr">
+        <is>
+          <t>Plyometric / Jump</t>
+        </is>
+      </c>
+      <c r="E268" s="7" t="inlineStr">
+        <is>
+          <t>Loaded triple-extension power with a low technical demand — the entry point into jump/Olympic-lift-pattern loading for athletes who aren't ready for a barbell variation yet</t>
+        </is>
+      </c>
+      <c r="F268" s="7" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="G268" s="7" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly, Low-Ceiling Friendly</t>
+        </is>
+      </c>
+      <c r="H268" s="7" t="inlineStr">
+        <is>
+          <t>Hold the dumbbells at your sides, load the hips, and jump straight up as high as you can — land soft and reset each rep, don't rush into the next one.</t>
+        </is>
+      </c>
+      <c r="I268" s="7" t="inlineStr">
+        <is>
+          <t>PJ-009 (Squat Jump, In Place)</t>
+        </is>
+      </c>
+      <c r="J268" s="7" t="inlineStr">
+        <is>
+          <t>PJ-029 (Trap Bar Jump)</t>
+        </is>
+      </c>
+      <c r="K268" s="7" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L268" s="7" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M268" s="7" t="n"/>
+      <c r="N268" s="7" t="n"/>
+      <c r="O268" s="7" t="inlineStr">
+        <is>
+          <t>Technical-coordination slot on Lower Body Strength Day and Impulse Day for athletes new to training (see day-structure-templates-spec: Olympic-lift gating) — a loaded jump pattern without the Olympic lift's catch/receiving position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="7" t="inlineStr">
+        <is>
+          <t>PJ-029</t>
+        </is>
+      </c>
+      <c r="B269" s="7" t="inlineStr">
+        <is>
+          <t>Trap Bar Jump</t>
+        </is>
+      </c>
+      <c r="C269" s="7" t="inlineStr">
+        <is>
+          <t>Core 50</t>
+        </is>
+      </c>
+      <c r="D269" s="7" t="inlineStr">
+        <is>
+          <t>Plyometric / Jump</t>
+        </is>
+      </c>
+      <c r="E269" s="7" t="inlineStr">
+        <is>
+          <t>Loaded triple-extension power at a higher load than a dumbbell allows, still without a catch/receiving position to coach</t>
+        </is>
+      </c>
+      <c r="F269" s="7" t="inlineStr">
+        <is>
+          <t>Trap Bar</t>
+        </is>
+      </c>
+      <c r="G269" s="7" t="inlineStr">
+        <is>
+          <t>Low-Ceiling Friendly</t>
+        </is>
+      </c>
+      <c r="H269" s="7" t="inlineStr">
+        <is>
+          <t>Set up like a trap bar deadlift, then explode up through the floor and jump — land soft back in the same stance and reset before the next rep.</t>
+        </is>
+      </c>
+      <c r="I269" s="7" t="inlineStr">
+        <is>
+          <t>PJ-028 (DB Jump)</t>
+        </is>
+      </c>
+      <c r="J269" s="7" t="inlineStr">
+        <is>
+          <t>OL-003 (Dumbbell Hang Clean)</t>
+        </is>
+      </c>
+      <c r="K269" s="7" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L269" s="7" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M269" s="7" t="n"/>
+      <c r="N269" s="7" t="n"/>
+      <c r="O269" s="7" t="inlineStr">
+        <is>
+          <t>Technical-coordination slot on Lower Body Strength Day and Impulse Day for athletes new to training (see day-structure-templates-spec: Olympic-lift gating) — bridges DB Jump up to the loads an Olympic-lift variation would use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>PJ-030</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>SL Hops — Lateral/Lateral/Medial/Medial (Continuous)</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Single-Leg / Ankle</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>Continuous single-leg frontal-plane reactive strength — repeated direction changes on one leg without resetting between reps</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>Hop laterally, laterally, then medially, medially, all on the same leg, continuously — quick ground contacts, stay stacked over the landing foot each time.</t>
+        </is>
+      </c>
+      <c r="I270" s="2" t="inlineStr">
+        <is>
+          <t>PJ-015 (Single-Leg Lateral Hop, Side-to-Side)</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="n"/>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L270" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M270" s="2" t="inlineStr">
+        <is>
+          <t>ankle injury-prevention relevant</t>
+        </is>
+      </c>
+      <c r="N270" s="2" t="n"/>
+      <c r="O270" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, middle phases — continuous multidirectional single-leg hopping for speed, once the hurdle-hop/stick-landing regressions are solid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>PJ-031</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>SL Hops — Fwd/Fwd/Bkwd/Bkwd (Continuous)</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Single-Leg / Ankle</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>Continuous single-leg sagittal-plane reactive strength — repeated direction changes on one leg without resetting between reps</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>Hop forward, forward, then backward, backward, all on the same leg, continuously — quick ground contacts, stay stacked over the landing foot each time.</t>
+        </is>
+      </c>
+      <c r="I271" s="2" t="inlineStr">
+        <is>
+          <t>PJ-017 (Single-Leg Hop and Stick, Deceleration)</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="n"/>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L271" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M271" s="2" t="inlineStr">
+        <is>
+          <t>ankle injury-prevention relevant</t>
+        </is>
+      </c>
+      <c r="N271" s="2" t="n"/>
+      <c r="O271" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, middle phases — continuous multidirectional single-leg hopping for speed, once the hurdle-hop/stick-landing regressions are solid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>PJ-032</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>SL Lateral/Medial Hurdle Hops — Stick Landing</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Single-Leg / Ankle</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg frontal-plane hop over a hurdle with a controlled, balanced landing — the entry point into multidirectional single-leg hopping</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>Mini Hurdles or Cones</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>Hop laterally then medially over the hurdle on one leg — land and freeze each time before the next hop. If you wobble, that's the rep telling you to slow down.</t>
+        </is>
+      </c>
+      <c r="I272" s="2" t="inlineStr">
+        <is>
+          <t>PJ-015 (Single-Leg Lateral Hop, Side-to-Side)</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>PJ-030 (SL Hops — Lateral/Lateral/Medial/Medial, Continuous)</t>
+        </is>
+      </c>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L272" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M272" s="2" t="inlineStr">
+        <is>
+          <t>ankle and ACL/knee injury-prevention relevant</t>
+        </is>
+      </c>
+      <c r="N272" s="2" t="n"/>
+      <c r="O272" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, early phases — controlled-landing single-leg multidirectional hopping is the early-phase version of the COD progression that continues into resisted lateral bounds and true COD sprinting/agility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>PJ-033</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>SL Fwd/Bkwd Hurdle Hops — Stick Landing</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Single-Leg / Ankle</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg sagittal-plane hop over a hurdle with a controlled, balanced landing — the entry point into multidirectional single-leg hopping</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>Mini Hurdles or Cones</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>Hop forward then backward over the hurdle on one leg — land and freeze each time before the next hop. If you wobble, that's the rep telling you to slow down.</t>
+        </is>
+      </c>
+      <c r="I273" s="2" t="inlineStr">
+        <is>
+          <t>PJ-017 (Single-Leg Hop and Stick, Deceleration)</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>PJ-031 (SL Hops — Fwd/Fwd/Bkwd/Bkwd, Continuous)</t>
+        </is>
+      </c>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L273" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M273" s="2" t="inlineStr">
+        <is>
+          <t>ankle and ACL/knee injury-prevention relevant</t>
+        </is>
+      </c>
+      <c r="N273" s="2" t="n"/>
+      <c r="O273" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, early phases — controlled-landing single-leg multidirectional hopping is the early-phase version of the COD progression that continues into resisted lateral bounds and true COD sprinting/agility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>PJ-034</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>Resisted Lateral Bound</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric / Jump</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>Frontal-plane power for cutting and marking, loaded with band resistance for extra force demand</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly, Low-Ceiling Friendly</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>Same bound as the unloaded version, but fight the band's pull on the way across — push off hard and stick the landing before you bound back.</t>
+        </is>
+      </c>
+      <c r="I274" s="2" t="inlineStr">
+        <is>
+          <t>PJ-003 (Lateral Bound)</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="n"/>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L274" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M274" s="2" t="n"/>
+      <c r="N274" s="2" t="n"/>
+      <c r="O274" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, middle phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>CD-013</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>Resisted 3-Step Lateral Deceleration</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>Lateral deceleration mechanics against band resistance over a short, controlled approach</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="inlineStr">
+        <is>
+          <t>Take three lateral steps against the band, chopping them down as you decelerate — finish balanced and in control, not falling into the last step.</t>
+        </is>
+      </c>
+      <c r="I275" s="2" t="inlineStr">
+        <is>
+          <t>CD-005 (Lateral Shuffle, Confined Space)</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>CD-014 (Resisted 3-Step Lateral Deceleration to Shuffle)</t>
+        </is>
+      </c>
+      <c r="K275" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L275" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M275" s="2" t="n"/>
+      <c r="N275" s="2" t="n"/>
+      <c r="O275" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, early-to-middle phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>CD-014</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Resisted 3-Step Lateral Deceleration to Shuffle</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>Lateral deceleration against band resistance that transitions directly into a defensive shuffle — closer to the mark's actual in-game movement</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>Decelerate over three steps against the band, then flow straight into a shuffle — no pause at the bottom, the deceleration and the shuffle are one continuous motion.</t>
+        </is>
+      </c>
+      <c r="I276" s="2" t="inlineStr">
+        <is>
+          <t>CD-013 (Resisted 3-Step Lateral Deceleration)</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>CD-015 (Resisted Lateral Shuffle)</t>
+        </is>
+      </c>
+      <c r="K276" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L276" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M276" s="2" t="n"/>
+      <c r="N276" s="2" t="n"/>
+      <c r="O276" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, middle phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>CD-015</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Resisted Lateral Shuffle</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>Defensive lateral movement mechanics loaded with band resistance for extra force demand</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t>Same shuffle as the unloaded version — stay low, feet don't cross — but drive harder off the trail leg to fight through the band's pull.</t>
+        </is>
+      </c>
+      <c r="I277" s="2" t="inlineStr">
+        <is>
+          <t>CD-005 (Lateral Shuffle, Confined Space)</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="n"/>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L277" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M277" s="2" t="n"/>
+      <c r="N277" s="2" t="n"/>
+      <c r="O277" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, middle phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>PJ-035</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>SL Continuous Hurdle Hops</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Single-Leg / Ankle</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>Continuous single-leg reactive strength over hurdles — rhythm and ground-contact time on one leg, without resetting between reps</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>Mini Hurdles or Cones</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>Quick ground contacts over each hurdle on one leg — 'hot coals,' minimal time on the floor. Stay tall and don't let the landing leg collapse.</t>
+        </is>
+      </c>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>PJ-032 (SL Lateral/Medial Hurdle Hops, Stick Landing)</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="n"/>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>ankle injury-prevention relevant</t>
+        </is>
+      </c>
+      <c r="N278" s="2" t="n"/>
+      <c r="O278" s="2" t="inlineStr">
+        <is>
+          <t>COD slot on Athlete Day, middle-to-late phases — the continuous-rhythm version of the stick-landing hurdle hop regressions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>SM-013</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>Band Resisted High Knees (In Place)</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>Sprint Mechanics</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>Sprint knee-drive patterning loaded with band resistance, without needing distance to run</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t>Drive the knees up fast against the band resistance — quick, light contacts, stay tall through the torso.</t>
+        </is>
+      </c>
+      <c r="I279" s="2" t="inlineStr">
+        <is>
+          <t>SM-009 (High Knees in Place)</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>SM-006 (Resisted Sprint, Sled Push/Pull)</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L279" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M279" s="2" t="n"/>
+      <c r="N279" s="2" t="n"/>
+      <c r="O279" s="2" t="inlineStr">
+        <is>
+          <t>Acceleration slot on Athlete Day for athletes with limited training space, or as early-phase acceleration work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>SM-014</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>Band Resisted A-Skips (In Place)</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>Sprint Mechanics</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>Knee drive and ground-contact patterning loaded with band resistance, without needing distance to run</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>Same A-skip pattern — drive the knee up, punch it down — but fight the band's pull on every rep. Quick and rhythmic, not slow and grinding.</t>
+        </is>
+      </c>
+      <c r="I280" s="2" t="inlineStr">
+        <is>
+          <t>SM-003 (A-Skip)</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>SM-006 (Resisted Sprint, Sled Push/Pull)</t>
+        </is>
+      </c>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L280" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M280" s="2" t="n"/>
+      <c r="N280" s="2" t="n"/>
+      <c r="O280" s="2" t="inlineStr">
+        <is>
+          <t>Acceleration slot on Athlete Day for athletes with limited training space, or as early-phase acceleration work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>SM-015</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Skips for Height</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>Sprint Mechanics</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>Vertical power expression of the skip pattern — bridges sprint-mechanics drilling into true plyometric output</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (10 yd)</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t>Skip forward but drive the lead knee up as high as you can each rep — maximum height, not speed down the line.</t>
+        </is>
+      </c>
+      <c r="I281" s="2" t="inlineStr">
+        <is>
+          <t>SM-003 (A-Skip)</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="n"/>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L281" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M281" s="2" t="n"/>
+      <c r="N281" s="2" t="n"/>
+      <c r="O281" s="2" t="inlineStr">
+        <is>
+          <t>Speed/acceleration slot on Athlete Day, middle-to-late phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>SM-016</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Skips for Distance</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>Sprint Mechanics</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>Horizontal power expression of the skip pattern — bridges sprint-mechanics drilling into true plyometric output</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (10 yd)</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr">
+        <is>
+          <t>Skip forward driving for maximum distance each rep — full extension and a strong arm swing, not a quick choppy skip.</t>
+        </is>
+      </c>
+      <c r="I282" s="2" t="inlineStr">
+        <is>
+          <t>SM-003 (A-Skip)</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="n"/>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L282" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M282" s="2" t="n"/>
+      <c r="N282" s="2" t="n"/>
+      <c r="O282" s="2" t="inlineStr">
+        <is>
+          <t>Speed/acceleration slot on Athlete Day, middle-to-late phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>PJ-036</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Kneeling Plyometric Push-Up</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Upper Body</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>Beginner entry into upper-body plyometric pressing — the kneeling position shortens the lever arm so the explosive push-off pattern can be learned before loading the full plank</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>None (Bodyweight)</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>Set up in a kneeling push-up position, brace, and push yourself explosively up off the ground — land soft with a slight bend in the elbows, same as the full version just from the knees.</t>
+        </is>
+      </c>
+      <c r="I283" s="2" t="n"/>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>PJ-037 (Band-Assisted Plyometric Push-Up)</t>
+        </is>
+      </c>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L283" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M283" s="2" t="n"/>
+      <c r="N283" s="2" t="n"/>
+      <c r="O283" s="2" t="inlineStr">
+        <is>
+          <t>Upper-body technical-coordination slot on Upper Body Strength Day and Hypertrophy Day for athletes new to training — the beginner on-ramp into the plyo push-up progression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>PJ-037</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Band-Assisted Plyometric Push-Up</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Upper Body</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>Beginner entry into upper-body plyometric pressing from a full plank — an overhead band offloads bodyweight so the explosive push-off pattern can be trained at full body length</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>Band, Anchor Point (Overhead)</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>Set up in a push-up with the band supporting you from overhead, brace, and push yourself explosively off the ground — land soft with a slight bend in the elbows. Let the band take the weight you're not ready for yet.</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>PJ-036 (Kneeling Plyometric Push-Up)</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>PJ-021 (Plyometric Push-Up, Clap Push-Up)</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L284" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M284" s="2" t="n"/>
+      <c r="N284" s="2" t="n"/>
+      <c r="O284" s="2" t="inlineStr">
+        <is>
+          <t>Upper-body technical-coordination slot on Upper Body Strength Day and Hypertrophy Day for athletes new to training — bridges the kneeling regression up to the full plyo push-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>PJ-038</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Kneeling Dumbbell Push Press</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Upper Body</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>Beginner entry into explosive overhead pressing — the kneeling (tall-kneeling) position removes the leg drive so the athlete learns to transfer trunk/arm explosiveness without needing push-press timing yet</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="n"/>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>Kneel tall, dumbbells at shoulder height, brace the core so you can't rock back — drive them overhead explosively and catch the lockout under control.</t>
+        </is>
+      </c>
+      <c r="I285" s="2" t="n"/>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>UP-001 (Push Press)</t>
+        </is>
+      </c>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L285" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M285" s="2" t="n"/>
+      <c r="N285" s="2" t="n"/>
+      <c r="O285" s="2" t="inlineStr">
+        <is>
+          <t>Upper-body technical-coordination slot on Upper Body Strength Day for athletes new to training — the beginner-friendly stand-in for a jerk/push-press variation until the athlete is ready for the standing, leg-driven version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>CR-034</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Weighted Sit-Up</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>Core - Anti-Extension</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>Advanced loaded crunch-pattern core work — higher-intensity option in the sagittal-plane core slot once bodyweight control is established</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbell or Weight Plate</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>Hold the weight at your chest, sit all the way up under control, and lower back down without letting it yank you — own the weight the whole rep, don't let it own you.</t>
+        </is>
+      </c>
+      <c r="I286" s="2" t="n"/>
+      <c r="J286" s="2" t="n"/>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L286" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M286" s="2" t="n"/>
+      <c r="N286" s="2" t="n"/>
+      <c r="O286" s="2" t="inlineStr">
+        <is>
+          <t>Crunch-variation slot in Lower Body Strength Day's secondary-pattern core superset (and Upper Body Strength Day's rotational/sagittal core pairing) — the advanced-tier option alongside CR-028 (Dead Bug with Plate Pass).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Library review: apply retire/edit decisions, add Run/Bike/Row conditioning interval ladder
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exercise Library'!$A$1:$Q$286</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exercise Library'!$A$1:$Q$302</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q286"/>
+  <dimension ref="A1:Q302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Push-Up (progression series)</t>
+          <t>Push-Ups</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -2686,7 +2686,7 @@
       <c r="P33" s="7" t="n"/>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -2727,11 +2727,7 @@
           <t>Load into your back hip, then whip the ball across your body into the wall — this should feel explosive, like you're throwing a punch with your whole torso.</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
-        <is>
-          <t>CR-001</t>
-        </is>
-      </c>
+      <c r="I34" s="7" t="n"/>
       <c r="J34" s="7" t="inlineStr"/>
       <c r="K34" s="7" t="inlineStr">
         <is>
@@ -3207,11 +3203,7 @@
           <t>Load quick, swing the arms, and explode up onto the box — land soft with the knees bent, don't just jump up and let it slam.</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr">
-        <is>
-          <t>IM-001 (Isometric hold at landing position)</t>
-        </is>
-      </c>
+      <c r="I42" s="7" t="n"/>
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>PJ-002</t>
@@ -3717,7 +3709,7 @@
       <c r="P50" s="2" t="n"/>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3721,7 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Acceleration Mechanics Drill (e.g., wall drill, falling starts)</t>
+          <t>Acceleration Mechanics Drill (e.g., wall drill)</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
@@ -4248,7 +4240,7 @@
       <c r="P59" s="2" t="n"/>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4358,7 @@
       <c r="P61" s="2" t="n"/>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4421,7 @@
       <c r="P62" s="2" t="n"/>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4543,7 @@
       <c r="P64" s="2" t="n"/>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4610,7 @@
       <c r="P65" s="2" t="n"/>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -4726,11 +4718,7 @@
           <t>Brace the hips up and curl the heels in under you — keep the hips high the whole set, don't let them sag toward the floor.</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>IS-001</t>
-        </is>
-      </c>
+      <c r="I67" s="2" t="n"/>
       <c r="J67" s="2" t="inlineStr">
         <is>
           <t>IS-003</t>
@@ -4815,7 +4803,7 @@
       <c r="P68" s="2" t="n"/>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -4856,11 +4844,7 @@
           <t>Keep a straight line from knees to shoulders and lean back slowly, using the quads to control the descent — this is a controlled lean, not a fall.</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>IS-005</t>
-        </is>
-      </c>
+      <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="inlineStr"/>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -5134,7 +5118,7 @@
       <c r="P73" s="7" t="n"/>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -5486,11 +5470,7 @@
           <t>Brace the side plank position, then squeeze the ball or bench between your legs as hard as you can and hold — the top knee should barely move.</t>
         </is>
       </c>
-      <c r="I79" s="7" t="inlineStr">
-        <is>
-          <t>IS-018</t>
-        </is>
-      </c>
+      <c r="I79" s="7" t="n"/>
       <c r="J79" s="7" t="inlineStr"/>
       <c r="K79" s="7" t="inlineStr">
         <is>
@@ -5650,7 +5630,7 @@
       <c r="P81" s="2" t="n"/>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -5662,7 +5642,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Glute Bridge (Bodyweight or Barbell)</t>
+          <t>Glute Bridge</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -5682,7 +5662,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>None or Barbell</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
@@ -5835,7 +5815,7 @@
       <c r="P84" s="2" t="n"/>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6272,7 @@
       <c r="P91" s="2" t="n"/>
       <c r="Q91" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -6713,7 +6693,7 @@
       <c r="P98" s="2" t="n"/>
       <c r="Q98" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6752,7 @@
       <c r="P99" s="2" t="n"/>
       <c r="Q99" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -6965,7 +6945,7 @@
       <c r="P102" s="2" t="n"/>
       <c r="Q102" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -7327,7 +7307,7 @@
       <c r="P108" s="2" t="n"/>
       <c r="Q108" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -7440,11 +7420,7 @@
           <t>UP-007</t>
         </is>
       </c>
-      <c r="J110" s="2" t="inlineStr">
-        <is>
-          <t>UP-011</t>
-        </is>
-      </c>
+      <c r="J110" s="2" t="n"/>
       <c r="K110" s="2" t="inlineStr">
         <is>
           <t>Novice</t>
@@ -7524,7 +7500,7 @@
       <c r="P111" s="2" t="n"/>
       <c r="Q111" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -7587,7 +7563,7 @@
       <c r="P112" s="2" t="n"/>
       <c r="Q112" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8166,7 +8142,7 @@
       <c r="P121" s="2" t="n"/>
       <c r="Q121" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8221,7 +8197,7 @@
       <c r="P122" s="7" t="n"/>
       <c r="Q122" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8280,7 +8256,7 @@
       <c r="P123" s="2" t="n"/>
       <c r="Q123" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8319,7 @@
       <c r="P124" s="2" t="n"/>
       <c r="Q124" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8406,7 +8382,7 @@
       <c r="P125" s="2" t="n"/>
       <c r="Q125" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8461,7 +8437,7 @@
       <c r="P126" s="2" t="n"/>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8520,7 +8496,7 @@
       <c r="P127" s="2" t="n"/>
       <c r="Q127" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8559,7 @@
       <c r="P128" s="2" t="n"/>
       <c r="Q128" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8646,7 +8622,7 @@
       <c r="P129" s="2" t="n"/>
       <c r="Q129" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8709,7 +8685,7 @@
       <c r="P130" s="2" t="n"/>
       <c r="Q130" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8772,7 +8748,7 @@
       <c r="P131" s="2" t="n"/>
       <c r="Q131" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8831,7 +8807,7 @@
       <c r="P132" s="2" t="n"/>
       <c r="Q132" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8890,7 +8866,7 @@
       <c r="P133" s="2" t="n"/>
       <c r="Q133" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -8902,7 +8878,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Steady-State Run/Bike/Row (20-40 min)</t>
+          <t>Run/Bike/Row — Steady State (20-60 min)</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -8922,12 +8898,12 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>None or Bike/Rower</t>
+          <t>None (Run), Bike, or Rower</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Confined Space Friendly (if machine-based)</t>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
         </is>
       </c>
       <c r="H134" s="11" t="inlineStr">
@@ -8936,7 +8912,11 @@
         </is>
       </c>
       <c r="I134" s="2" t="inlineStr"/>
-      <c r="J134" s="2" t="inlineStr"/>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>CN-033</t>
+        </is>
+      </c>
       <c r="K134" s="2" t="inlineStr">
         <is>
           <t>Novice</t>
@@ -8944,12 +8924,16 @@
       </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
-          <t>Off-season</t>
+          <t>Off-season, Pre-season</t>
         </is>
       </c>
       <c r="M134" s="2" t="inlineStr"/>
       <c r="N134" s="2" t="inlineStr"/>
-      <c r="O134" s="2" t="n"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>Zone 2 continuous, RPE 4-5 (talk-test: full sentences). Dose by phase — GPP/Reacclimation: 40-60 min; Hypertrophy: 30-45 min; Max Strength: 20-30 min; Power Conversion / Peak: 20-30 min as recovery only; in-season: 20-30 min optional. Run: steady jog. Bike/Row: steady cadence/split.</t>
+        </is>
+      </c>
       <c r="P134" s="2" t="n"/>
       <c r="Q134" s="2" t="inlineStr">
         <is>
@@ -9012,7 +8996,7 @@
       <c r="P135" s="7" t="n"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -9075,7 +9059,7 @@
       <c r="P136" s="2" t="n"/>
       <c r="Q136" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9122,7 @@
       <c r="P137" s="2" t="n"/>
       <c r="Q137" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -9209,7 +9193,7 @@
       <c r="P138" s="2" t="n"/>
       <c r="Q138" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9619,7 @@
       <c r="P144" s="2" t="n"/>
       <c r="Q144" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -9970,7 +9954,7 @@
       <c r="P149" s="2" t="n"/>
       <c r="Q149" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -10480,11 +10464,7 @@
           <t>Hop out and land on one leg — the moment your foot touches, freeze and hold it. If you wobble or need a second hop to balance, that's the rep giving you feedback.</t>
         </is>
       </c>
-      <c r="I157" s="7" t="inlineStr">
-        <is>
-          <t>IM-008</t>
-        </is>
-      </c>
+      <c r="I157" s="7" t="n"/>
       <c r="J157" s="7" t="inlineStr">
         <is>
           <t>PJ-016</t>
@@ -13028,11 +13008,7 @@
           <t>Half-kneeling so you can't cheat with your hips — press the band straight out and hold, resisting any rotation through the torso.</t>
         </is>
       </c>
-      <c r="I197" s="2" t="inlineStr">
-        <is>
-          <t>CR-001</t>
-        </is>
-      </c>
+      <c r="I197" s="2" t="n"/>
       <c r="J197" s="2" t="inlineStr">
         <is>
           <t>CR-014</t>
@@ -13099,11 +13075,7 @@
           <t>Press the band out and hold your center, then march in place without letting your torso twist toward the band. Slow and controlled beats fast and sloppy.</t>
         </is>
       </c>
-      <c r="I198" s="2" t="inlineStr">
-        <is>
-          <t>CR-001</t>
-        </is>
-      </c>
+      <c r="I198" s="2" t="n"/>
       <c r="J198" s="2" t="inlineStr"/>
       <c r="K198" s="2" t="inlineStr">
         <is>
@@ -13444,7 +13416,7 @@
       <c r="P203" s="2" t="n"/>
       <c r="Q203" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -13893,7 +13865,7 @@
       <c r="P210" s="2" t="n"/>
       <c r="Q210" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -14575,7 +14547,7 @@
       <c r="P220" s="9" t="n"/>
       <c r="Q220" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -14692,11 +14664,7 @@
         </is>
       </c>
       <c r="I222" s="9" t="n"/>
-      <c r="J222" s="9" t="inlineStr">
-        <is>
-          <t>IM-001</t>
-        </is>
-      </c>
+      <c r="J222" s="9" t="n"/>
       <c r="K222" s="9" t="inlineStr">
         <is>
           <t>Novice</t>
@@ -14758,11 +14726,7 @@
           <t>Set the front knee at the target angle and hold — steady pressure through the front foot, this one tests your balance as much as your strength.</t>
         </is>
       </c>
-      <c r="I223" s="9" t="inlineStr">
-        <is>
-          <t>IM-001</t>
-        </is>
-      </c>
+      <c r="I223" s="9" t="n"/>
       <c r="J223" s="9" t="inlineStr"/>
       <c r="K223" s="9" t="inlineStr">
         <is>
@@ -15056,7 +15020,7 @@
       <c r="P227" s="9" t="n"/>
       <c r="Q227" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -15328,7 +15292,7 @@
       <c r="P231" s="9" t="n"/>
       <c r="Q231" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -15395,7 +15359,7 @@
       <c r="P232" s="9" t="n"/>
       <c r="Q232" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -15667,7 +15631,7 @@
       <c r="P236" s="9" t="n"/>
       <c r="Q236" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -15738,7 +15702,7 @@
       <c r="P237" s="9" t="n"/>
       <c r="Q237" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -15821,7 +15785,7 @@
       </c>
       <c r="B239" s="9" t="inlineStr">
         <is>
-          <t>Kettlebell Swing (Russian)</t>
+          <t>Kettlebell Swing</t>
         </is>
       </c>
       <c r="C239" s="9" t="inlineStr">
@@ -16830,7 +16794,7 @@
       <c r="P253" s="9" t="n"/>
       <c r="Q253" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -16893,7 +16857,7 @@
       <c r="P254" s="9" t="n"/>
       <c r="Q254" s="9" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -16950,7 +16914,7 @@
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17012,7 +16976,7 @@
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17074,7 +17038,7 @@
       </c>
       <c r="Q257" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17114,16 +17078,6 @@
           <t>Stay low in the backpedal, then snap the hips and drive forward the instant you flip — the transition should be one motion, not two.</t>
         </is>
       </c>
-      <c r="I258" t="inlineStr">
-        <is>
-          <t>CD-005</t>
-        </is>
-      </c>
-      <c r="J258" t="inlineStr">
-        <is>
-          <t>CD-006</t>
-        </is>
-      </c>
       <c r="K258" t="inlineStr">
         <is>
           <t>Both</t>
@@ -17193,7 +17147,7 @@
       </c>
       <c r="Q259" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17255,7 +17209,7 @@
       </c>
       <c r="Q260" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17317,7 +17271,7 @@
       </c>
       <c r="Q261" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17388,7 +17342,7 @@
       <c r="P262" s="7" t="n"/>
       <c r="Q262" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -17433,11 +17387,7 @@
           <t>Bound laterally like before, but this time finish by driving straight up into a stick — redirect the momentum from sideways to vertical without losing your landing control.</t>
         </is>
       </c>
-      <c r="I263" s="2" t="inlineStr">
-        <is>
-          <t>RS-001</t>
-        </is>
-      </c>
+      <c r="I263" s="2" t="n"/>
       <c r="J263" s="2" t="inlineStr">
         <is>
           <t>RS-003</t>
@@ -17538,7 +17488,7 @@
       </c>
       <c r="B265" s="7" t="inlineStr">
         <is>
-          <t>KB Loaded Deceleration Step (Entry)</t>
+          <t>Band Loaded Deceleration Step (Entry)</t>
         </is>
       </c>
       <c r="C265" s="7" t="inlineStr">
@@ -17558,7 +17508,7 @@
       </c>
       <c r="F265" s="7" t="inlineStr">
         <is>
-          <t>Kettlebell</t>
+          <t>Bands</t>
         </is>
       </c>
       <c r="G265" s="7" t="inlineStr">
@@ -17568,7 +17518,7 @@
       </c>
       <c r="H265" s="7" t="inlineStr">
         <is>
-          <t>Hold the kettlebell at your chest, take two building steps, then plant hard and stick a low, balanced stance — the goal is stopping on a dime, not drifting through the landing.</t>
+          <t>Loop a band around your hips, anchored low behind you. Take two building steps against the band tension, then plant hard and stick a low, balanced stance — the band is trying to pull you off balance, so the goal is stopping on a dime, not drifting through the landing.</t>
         </is>
       </c>
       <c r="I265" s="7" t="n"/>
@@ -17605,7 +17555,7 @@
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>KB Loaded Deceleration Step to Reactive Redirect</t>
+          <t>Band Loaded Deceleration Step to Reactive Redirect</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
@@ -17625,7 +17575,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>Kettlebell</t>
+          <t>Bands</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -17643,11 +17593,7 @@
           <t>RS-004</t>
         </is>
       </c>
-      <c r="J266" s="2" t="inlineStr">
-        <is>
-          <t>RS-006</t>
-        </is>
-      </c>
+      <c r="J266" s="2" t="n"/>
       <c r="K266" s="2" t="inlineStr">
         <is>
           <t>Both</t>
@@ -17731,7 +17677,7 @@
       <c r="P267" s="2" t="n"/>
       <c r="Q267" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -18297,11 +18243,7 @@
           <t>Take three lateral steps against the band, chopping them down as you decelerate — finish balanced and in control, not falling into the last step.</t>
         </is>
       </c>
-      <c r="I275" s="2" t="inlineStr">
-        <is>
-          <t>CD-005 (Lateral Shuffle, Confined Space)</t>
-        </is>
-      </c>
+      <c r="I275" s="2" t="n"/>
       <c r="J275" s="2" t="inlineStr">
         <is>
           <t>CD-014 (Resisted 3-Step Lateral Deceleration to Shuffle)</t>
@@ -18447,11 +18389,7 @@
           <t>Same shuffle as the unloaded version — stay low, feet don't cross — but drive harder off the trail leg to fight through the band's pull.</t>
         </is>
       </c>
-      <c r="I277" s="2" t="inlineStr">
-        <is>
-          <t>CD-005 (Lateral Shuffle, Confined Space)</t>
-        </is>
-      </c>
+      <c r="I277" s="2" t="n"/>
       <c r="J277" s="2" t="n"/>
       <c r="K277" s="2" t="inlineStr">
         <is>
@@ -19116,8 +19054,1172 @@
         </is>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>CN-018</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Max Sprints (5-10s)</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Alactic / Speed</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>Pure alactic (ATP-PC) power: the shortest all-out efforts, trained fresh with full recovery.</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H287" s="11" t="inlineStr">
+        <is>
+          <t>All-out from the first second — this is a sprint, not a pace. Stop the moment the clock says go home, then fully recover; if the last rep isn't as fast as the first, we're done.</t>
+        </is>
+      </c>
+      <c r="I287" s="2" t="n"/>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>CN-019</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L287" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M287" s="2" t="n"/>
+      <c r="N287" s="2" t="n"/>
+      <c r="O287" s="2" t="inlineStr">
+        <is>
+          <t>Work 5-10s max effort | Rest 60-90s (about 1:10) | 6-10 reps, 1 block. Quality-gated: stop when output drops ~5-10%. Run: 10-30 yd sprint, walk back. Bike: assault/spin bike, seated or standing, max watts. Row: 5-8 hard strokes at max power. RPE 10.</t>
+        </is>
+      </c>
+      <c r="P287" s="2" t="n"/>
+      <c r="Q287" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>CN-019</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Power Intervals (10-15s)</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Alactic / Speed</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>Alactic power with a little glycolytic spillover; the classic "short burst" interval.</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H288" s="11" t="inlineStr">
+        <is>
+          <t>Max effort, every rep — the first 5 seconds should feel violent, and you hold on for the rest. Rest means rest: walk, breathe, and come back fresh.</t>
+        </is>
+      </c>
+      <c r="I288" s="2" t="inlineStr">
+        <is>
+          <t>CN-018</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>CN-020</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L288" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M288" s="2" t="n"/>
+      <c r="N288" s="2" t="n"/>
+      <c r="O288" s="2" t="inlineStr">
+        <is>
+          <t>Work 10-15s max effort | Rest 90-120s (about 1:8) | 6-8 reps. Run: 40-80 yd. Bike: 10-15s all-out. Row: 10-15s, around 8-12 strokes. RPE 10.</t>
+        </is>
+      </c>
+      <c r="P288" s="2" t="n"/>
+      <c r="Q288" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>CN-020</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Speed Intervals (15-20s)</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Alactic / Speed</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>Top of the alactic window: sustaining maximal output as the phosphocreatine system starts to run down.</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H289" s="11" t="inlineStr">
+        <is>
+          <t>Attack the whole interval — don't pace the first half, and keep your form clean as it gets hard. Full recovery between reps so every one counts.</t>
+        </is>
+      </c>
+      <c r="I289" s="2" t="inlineStr">
+        <is>
+          <t>CN-019</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="n"/>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L289" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M289" s="2" t="n"/>
+      <c r="N289" s="2" t="n"/>
+      <c r="O289" s="2" t="inlineStr">
+        <is>
+          <t>Work 15-20s max effort | Rest 2-3 min (about 1:8) | 4-6 reps. Run: 100-150 yd. Bike: 15-20s all-out. Row: 15-20s, about 14-18 strokes. RPE 9-10. Advanced because the end of the interval carries real fatigue.</t>
+        </is>
+      </c>
+      <c r="P289" s="2" t="n"/>
+      <c r="Q289" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>CN-021</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Repeated Sprints (5-10s on / 20-30s off)</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Repeated Sprint Ability</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>Repeated-sprint ability: many short max efforts with incomplete recovery — the closest match to the cut-and-burst pattern of a point.</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H290" s="11" t="inlineStr">
+        <is>
+          <t>Every rep at max — the point is holding speed while the rest gets shorter than you want. If you can't hit speed anymore, end the set.</t>
+        </is>
+      </c>
+      <c r="I290" s="2" t="n"/>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>CN-022</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L290" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season, In-season</t>
+        </is>
+      </c>
+      <c r="M290" s="2" t="n"/>
+      <c r="N290" s="2" t="n"/>
+      <c r="O290" s="2" t="inlineStr">
+        <is>
+          <t>Work 5-10s max | Rest 20-30s | 6-10 reps per set, 2-3 sets, 3-4 min between sets. Run: 10-20 yd sprints with a quick jog or walk back. Bike: max-watt bursts. Row: 5-8 hard strokes. RPE 9-10.</t>
+        </is>
+      </c>
+      <c r="P290" s="2" t="n"/>
+      <c r="Q290" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>CN-022</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Repeated Sprints (10-15s on / 30-45s off)</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Repeated Sprint Ability</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>Longer repeated sprints with a game-realistic work:rest ratio; builds the ability to repeat high-intensity bursts across a tournament day.</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H291" s="11" t="inlineStr">
+        <is>
+          <t>Hard, honest sprints and honest rest — go hard when it's go time, actually recover when it's rest time. Hold the same speed on the last rep as the first.</t>
+        </is>
+      </c>
+      <c r="I291" s="2" t="inlineStr">
+        <is>
+          <t>CN-021</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>CN-023</t>
+        </is>
+      </c>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L291" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season, In-season</t>
+        </is>
+      </c>
+      <c r="M291" s="2" t="n"/>
+      <c r="N291" s="2" t="n"/>
+      <c r="O291" s="2" t="inlineStr">
+        <is>
+          <t>Work 10-15s | Rest 30-45s | 6-8 reps per set, 2-3 sets, 3-4 min between sets. Run: 30-60 yd sprints. Bike: hard 10-15s efforts. Row: 10-15s hard. RPE 9.</t>
+        </is>
+      </c>
+      <c r="P291" s="2" t="n"/>
+      <c r="Q291" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>CN-023</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Point Simulation (30-45s on / 45-60s off)</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Repeated Sprint Ability</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>Mimics an actual point (30-90s of intermittent high-intensity play) with game-like recovery between points.</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H292" s="11" t="inlineStr">
+        <is>
+          <t>Treat each round like a real point — surge, settle, surge again — and use the break to bring your breathing down. The last point should look like the first.</t>
+        </is>
+      </c>
+      <c r="I292" s="2" t="inlineStr">
+        <is>
+          <t>CN-022</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="n"/>
+      <c r="K292" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L292" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season, In-season</t>
+        </is>
+      </c>
+      <c r="M292" s="2" t="n"/>
+      <c r="N292" s="2" t="n"/>
+      <c r="O292" s="2" t="inlineStr">
+        <is>
+          <t>Work 30-45s as surges (e.g. 10s hard / 5s easy repeating) | Rest 45-60s | 5-7 rounds, 1-2 sets, 4-5 min between sets. Run: shuttle or straight-line surges. Bike: 10s hard / 5s easy. Row: 10s hard / 5s easy. RPE 8-9.</t>
+        </is>
+      </c>
+      <c r="P292" s="2" t="n"/>
+      <c r="Q292" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>CN-024</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Short Glycolytic Intervals (20-30s)</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Glycolytic / Anaerobic</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>Entry glycolytic (anaerobic) work: hard, short efforts that build buffering and speed-endurance without long lactate exposure.</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G293" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H293" s="11" t="inlineStr">
+        <is>
+          <t>Hard and controlled, about 90-95% — fast but not flailing. Hold your form to the end of every interval and use the full rest.</t>
+        </is>
+      </c>
+      <c r="I293" s="2" t="n"/>
+      <c r="J293" s="2" t="inlineStr">
+        <is>
+          <t>CN-025</t>
+        </is>
+      </c>
+      <c r="K293" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L293" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season</t>
+        </is>
+      </c>
+      <c r="M293" s="2" t="n"/>
+      <c r="N293" s="2" t="n"/>
+      <c r="O293" s="2" t="inlineStr">
+        <is>
+          <t>Work 20-30s at ~90-95% | Rest 90-150s (about 1:4-1:5) | 5-8 reps. Run: 150-200 yd. Bike: 20-30s hard. Row: 20-30s, about 18-24 strokes. RPE 8-9.</t>
+        </is>
+      </c>
+      <c r="P293" s="2" t="n"/>
+      <c r="Q293" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>CN-025</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Glycolytic Intervals (30-45s)</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Glycolytic / Anaerobic</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>Mid-range glycolytic capacity; the work length of a typical high-intensity stretch within a point.</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G294" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H294" s="11" t="inlineStr">
+        <is>
+          <t>Strong, even pace — start at a speed you can hold to the finish. It should hurt in the last third, and your form should still be there.</t>
+        </is>
+      </c>
+      <c r="I294" s="2" t="inlineStr">
+        <is>
+          <t>CN-024</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>CN-026</t>
+        </is>
+      </c>
+      <c r="K294" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L294" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season</t>
+        </is>
+      </c>
+      <c r="M294" s="2" t="n"/>
+      <c r="N294" s="2" t="n"/>
+      <c r="O294" s="2" t="inlineStr">
+        <is>
+          <t>Work 30-45s at ~90% | Rest 90-135s (about 1:3) | 4-6 reps. Run: 200-300 yd. Bike: 30-45s hard. Row: 30-45s hard, steady rate. RPE 8-9.</t>
+        </is>
+      </c>
+      <c r="P294" s="2" t="n"/>
+      <c r="Q294" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>CN-026</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Lactate Tolerance Intervals (45-60s)</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Glycolytic / Anaerobic</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>Builds tolerance to sustained high lactate; closes the gap between short bursts and aerobic power work.</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G295" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H295" s="11" t="inlineStr">
+        <is>
+          <t>Aggressive but controlled — go out hard, settle, and fight to hold the pace to the end. The last 10 seconds are the rep.</t>
+        </is>
+      </c>
+      <c r="I295" s="2" t="inlineStr">
+        <is>
+          <t>CN-025</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>CN-027</t>
+        </is>
+      </c>
+      <c r="K295" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L295" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season</t>
+        </is>
+      </c>
+      <c r="M295" s="2" t="n"/>
+      <c r="N295" s="2" t="n"/>
+      <c r="O295" s="2" t="inlineStr">
+        <is>
+          <t>Work 45-60s at ~90% | Rest 2-3 min (about 1:3) | 4-6 reps. Run: 300-400 yd (a 300-yd shuttle works). Bike: 45-60s hard. Row: 45-60s hard. RPE 9.</t>
+        </is>
+      </c>
+      <c r="P295" s="2" t="n"/>
+      <c r="Q295" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>CN-027</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Extended Glycolytic Intervals (60-90s)</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Glycolytic / Anaerobic</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>Top of the glycolytic range; overlaps into aerobic power and teaches pacing under heavy fatigue.</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G296" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H296" s="11" t="inlineStr">
+        <is>
+          <t>Smart start, strong finish — find a pace you can hold the whole interval, because the back half is where it gets decided. Rest fully so the next one is still quality.</t>
+        </is>
+      </c>
+      <c r="I296" s="2" t="inlineStr">
+        <is>
+          <t>CN-026</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="n"/>
+      <c r="K296" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L296" s="2" t="inlineStr">
+        <is>
+          <t>Pre-season</t>
+        </is>
+      </c>
+      <c r="M296" s="2" t="n"/>
+      <c r="N296" s="2" t="n"/>
+      <c r="O296" s="2" t="inlineStr">
+        <is>
+          <t>Work 60-90s at ~85-90% | Rest 3-4 min (about 1:2-1:3) | 3-5 reps. Run: 400-600 yd. Bike: 60-90s hard. Row: 60-90s hard. RPE 8-9.</t>
+        </is>
+      </c>
+      <c r="P296" s="2" t="n"/>
+      <c r="Q296" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>CN-028</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — 30/30 Intervals (30s on / 30s off)</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Aerobic Power</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>Aerobic power (VO2max): short hard intervals with equal rest keep oxygen uptake near max for long total time.</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G297" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H297" s="11" t="inlineStr">
+        <is>
+          <t>Hard but repeatable — about 90-95% of your top effort, and the same speed on the last interval as the first. Easy jog or spin in the 30s off, don't stop.</t>
+        </is>
+      </c>
+      <c r="I297" s="2" t="n"/>
+      <c r="J297" s="2" t="inlineStr">
+        <is>
+          <t>CN-029</t>
+        </is>
+      </c>
+      <c r="K297" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L297" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M297" s="2" t="n"/>
+      <c r="N297" s="2" t="n"/>
+      <c r="O297" s="2" t="inlineStr">
+        <is>
+          <t>Work 30s at ~90-95% | Rest 30s easy | 10-20 reps (1-2 blocks of 8-10, 3 min between blocks). Run: fast, smooth running. Bike: hard, repeatable cadence. Row: 30s steady hard rate. RPE 8.</t>
+        </is>
+      </c>
+      <c r="P297" s="2" t="n"/>
+      <c r="Q297" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>CN-029</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Aerobic Power Intervals (2 min)</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Aerobic Power</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="inlineStr">
+        <is>
+          <t>VO2max development with a manageable length; the rep you can repeat many times.</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G298" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H298" s="11" t="inlineStr">
+        <is>
+          <t>Controlled and strong from the start — a pace you could just barely hold for 3 minutes. Breathe in rhythm and keep your form.</t>
+        </is>
+      </c>
+      <c r="I298" s="2" t="inlineStr">
+        <is>
+          <t>CN-028</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>CN-030</t>
+        </is>
+      </c>
+      <c r="K298" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L298" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M298" s="2" t="n"/>
+      <c r="N298" s="2" t="n"/>
+      <c r="O298" s="2" t="inlineStr">
+        <is>
+          <t>Work 2 min at ~90-95% HRmax | Rest 2 min easy | 5-8 reps. Run: track or road, even pace. Bike: steady hard watts. Row: steady, low-to-mid stroke rate. RPE 8.</t>
+        </is>
+      </c>
+      <c r="P298" s="2" t="n"/>
+      <c r="Q298" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>CN-030</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Aerobic Power Intervals (3 min)</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Aerobic Power</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>VO2max intervals at a length where oxygen uptake is held near max for the whole rep.</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G299" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H299" s="11" t="inlineStr">
+        <is>
+          <t>Settle in by the first 30 seconds, then hold. You should finish thinking you had maybe one more minute — no more.</t>
+        </is>
+      </c>
+      <c r="I299" s="2" t="inlineStr">
+        <is>
+          <t>CN-029</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>CN-031</t>
+        </is>
+      </c>
+      <c r="K299" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L299" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M299" s="2" t="n"/>
+      <c r="N299" s="2" t="n"/>
+      <c r="O299" s="2" t="inlineStr">
+        <is>
+          <t>Work 3 min at ~90-95% HRmax | Rest 2-3 min easy | 4-6 reps. Run: even pace. Bike: steady hard watts. Row: steady hard split. RPE 8.</t>
+        </is>
+      </c>
+      <c r="P299" s="2" t="n"/>
+      <c r="Q299" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>CN-031</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Aerobic Power Intervals (4 min)</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Aerobic Power</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="inlineStr">
+        <is>
+          <t>The classic 4x4 aerobic power session; the most time near max oxygen uptake for a single interval length.</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G300" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H300" s="11" t="inlineStr">
+        <is>
+          <t>Even, strong pace the whole 4 minutes. Don't blow up in the first minute — the last minute should feel hard but still controlled.</t>
+        </is>
+      </c>
+      <c r="I300" s="2" t="inlineStr">
+        <is>
+          <t>CN-030</t>
+        </is>
+      </c>
+      <c r="J300" s="2" t="n"/>
+      <c r="K300" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L300" s="2" t="inlineStr">
+        <is>
+          <t>Off-season</t>
+        </is>
+      </c>
+      <c r="M300" s="2" t="n"/>
+      <c r="N300" s="2" t="n"/>
+      <c r="O300" s="2" t="inlineStr">
+        <is>
+          <t>Work 4 min at ~90-95% HRmax | Rest 3 min easy | 4 reps. Run: even pace. Bike: steady hard watts. Row: steady hard split. RPE 8-9.</t>
+        </is>
+      </c>
+      <c r="P300" s="2" t="n"/>
+      <c r="Q300" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>CN-032</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Threshold / Tempo Intervals (5-8 min)</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Aerobic Capacity</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>Aerobic capacity at the top of the aerobic range: comfortably-hard efforts that raise the pace you can hold for a long time.</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G301" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H301" s="11" t="inlineStr">
+        <is>
+          <t>Comfortably hard — you could talk in short phrases but wouldn't want to. Even splits, steady breathing.</t>
+        </is>
+      </c>
+      <c r="I301" s="2" t="inlineStr">
+        <is>
+          <t>CN-033</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="n"/>
+      <c r="K301" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L301" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M301" s="2" t="n"/>
+      <c r="N301" s="2" t="n"/>
+      <c r="O301" s="2" t="inlineStr">
+        <is>
+          <t>Work 5-8 min at ~80-85% HRmax | Rest 1-2 min easy | 3-5 reps. Run: even pace. Bike: steady cadence. Row: steady, controlled split. RPE 6-7.</t>
+        </is>
+      </c>
+      <c r="P301" s="2" t="n"/>
+      <c r="Q301" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>CN-033</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>Run/Bike/Row — Long Aerobic Intervals (10-15 min)</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>Conditioning - Aerobic Capacity</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>Bridges interval work and steady state: long, controlled aerobic efforts with short breaks.</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>None (Run), Bike, or Rower</t>
+        </is>
+      </c>
+      <c r="G302" s="2" t="inlineStr">
+        <is>
+          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+        </is>
+      </c>
+      <c r="H302" s="11" t="inlineStr">
+        <is>
+          <t>Easy-to-moderate and relaxed — hold the same pace the whole time, finishing feeling like you could do more.</t>
+        </is>
+      </c>
+      <c r="I302" s="2" t="inlineStr">
+        <is>
+          <t>CN-009</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>CN-032</t>
+        </is>
+      </c>
+      <c r="K302" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L302" s="2" t="inlineStr">
+        <is>
+          <t>Off-season</t>
+        </is>
+      </c>
+      <c r="M302" s="2" t="n"/>
+      <c r="N302" s="2" t="n"/>
+      <c r="O302" s="2" t="inlineStr">
+        <is>
+          <t>Work 10-15 min at ~70-80% HRmax | Rest 2-3 min easy | 2-3 reps. Run: steady run. Bike: steady spin. Row: steady rhythmic rowing. RPE 5-6.</t>
+        </is>
+      </c>
+      <c r="P302" s="2" t="n"/>
+      <c r="Q302" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q286"/>
+  <autoFilter ref="A1:Q302"/>
   <dataValidations count="6">
     <dataValidation sqref="C2:C900" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Core 50,Extended Library"</formula1>

</xml_diff>

<commit_message>
Library review: apply retire/edit decisions, Run/Bike/Row conditioning ladder, injury + season tag fixes, 18 new exercises
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exercise Library'!$A$1:$Q$302</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exercise Library'!$A$1:$Q$320</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q302"/>
+  <dimension ref="A1:Q320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1024,7 +1024,11 @@
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="7" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M8" s="7" t="inlineStr"/>
       <c r="N8" s="7" t="inlineStr"/>
       <c r="O8" s="7" t="inlineStr">
@@ -1091,7 +1095,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M9" s="7" t="inlineStr"/>
       <c r="N9" s="7" t="inlineStr"/>
       <c r="O9" s="7" t="n"/>
@@ -1154,7 +1162,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M10" s="7" t="inlineStr"/>
       <c r="N10" s="7" t="inlineStr"/>
       <c r="O10" s="7" t="n"/>
@@ -1221,7 +1233,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M11" s="7" t="inlineStr"/>
       <c r="N11" s="7" t="inlineStr"/>
       <c r="O11" s="7" t="n"/>
@@ -1292,7 +1308,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M12" s="7" t="inlineStr"/>
       <c r="N12" s="7" t="inlineStr"/>
       <c r="O12" s="7" t="n"/>
@@ -1359,7 +1379,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="n"/>
@@ -1422,7 +1446,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr"/>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M14" s="7" t="inlineStr"/>
       <c r="N14" s="7" t="inlineStr"/>
       <c r="O14" s="7" t="n"/>
@@ -1470,7 +1498,11 @@
           <t>Straight line from head to heels — squeeze the glutes so the hips don't sag. Chest to the floor, then push the ground away hard.</t>
         </is>
       </c>
-      <c r="I15" s="7" t="n"/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>UP-017</t>
+        </is>
+      </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
           <t>UP-003</t>
@@ -1556,7 +1588,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Shoulder-friendly pressing angle</t>
@@ -1619,7 +1655,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M17" s="7" t="inlineStr"/>
       <c r="N17" s="7" t="inlineStr"/>
       <c r="O17" s="7" t="n"/>
@@ -1678,7 +1718,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr"/>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="7" t="inlineStr"/>
       <c r="O18" s="7" t="n"/>
@@ -1808,7 +1852,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr"/>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M20" s="7" t="inlineStr"/>
       <c r="N20" s="7" t="inlineStr"/>
       <c r="O20" s="7" t="n"/>
@@ -2734,7 +2782,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L34" s="7" t="inlineStr"/>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M34" s="7" t="inlineStr"/>
       <c r="N34" s="7" t="inlineStr"/>
       <c r="O34" s="7" t="n"/>
@@ -2794,7 +2846,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M35" s="7" t="inlineStr"/>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N35" s="7" t="inlineStr"/>
       <c r="O35" s="7" t="n"/>
       <c r="P35" s="7" t="n"/>
@@ -2853,7 +2909,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="n"/>
@@ -2911,8 +2971,16 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="n"/>
@@ -2971,7 +3039,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="n"/>
@@ -3034,7 +3106,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M39" s="7" t="inlineStr"/>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N39" s="7" t="inlineStr"/>
       <c r="O39" s="7" t="n"/>
       <c r="P39" s="7" t="n"/>
@@ -3093,7 +3169,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M40" s="7" t="inlineStr"/>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N40" s="7" t="inlineStr"/>
       <c r="O40" s="7" t="n"/>
       <c r="P40" s="7" t="n"/>
@@ -3151,8 +3231,16 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="n"/>
@@ -3214,7 +3302,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr"/>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
           <t>Tendon-pain regression per Sec. 5</t>
@@ -3285,7 +3377,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L43" s="7" t="inlineStr"/>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
       <c r="M43" s="7" t="inlineStr"/>
       <c r="N43" s="7" t="inlineStr"/>
       <c r="O43" s="7" t="n"/>
@@ -3340,7 +3436,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L44" s="7" t="inlineStr"/>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M44" s="7" t="inlineStr"/>
       <c r="N44" s="7" t="inlineStr"/>
       <c r="O44" s="7" t="n"/>
@@ -3395,7 +3495,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="n"/>
@@ -3454,7 +3558,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="n"/>
@@ -3509,7 +3617,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L47" s="7" t="inlineStr"/>
+      <c r="L47" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M47" s="7" t="inlineStr"/>
       <c r="N47" s="7" t="inlineStr"/>
       <c r="O47" s="7" t="n"/>
@@ -3757,7 +3869,11 @@
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr"/>
-      <c r="L51" s="7" t="inlineStr"/>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M51" s="7" t="inlineStr"/>
       <c r="N51" s="7" t="inlineStr"/>
       <c r="O51" s="7" t="n"/>
@@ -3812,7 +3928,11 @@
       </c>
       <c r="J52" s="7" t="inlineStr"/>
       <c r="K52" s="7" t="inlineStr"/>
-      <c r="L52" s="7" t="inlineStr"/>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M52" s="7" t="inlineStr"/>
       <c r="N52" s="7" t="inlineStr"/>
       <c r="O52" s="7" t="n"/>
@@ -3997,7 +4117,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L55" s="7" t="inlineStr"/>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M55" s="7" t="inlineStr"/>
       <c r="N55" s="7" t="inlineStr"/>
       <c r="O55" s="7" t="n"/>
@@ -4060,7 +4184,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L56" s="7" t="inlineStr"/>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
       <c r="M56" s="7" t="inlineStr"/>
       <c r="N56" s="7" t="inlineStr"/>
       <c r="O56" s="7" t="n"/>
@@ -4123,7 +4251,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M57" s="2" t="inlineStr"/>
       <c r="N57" s="2" t="inlineStr"/>
       <c r="O57" s="2" t="n"/>
@@ -4182,7 +4314,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L58" s="7" t="inlineStr"/>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M58" s="7" t="inlineStr"/>
       <c r="N58" s="7" t="inlineStr"/>
       <c r="O58" s="7" t="n"/>
@@ -4292,7 +4428,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M60" s="2" t="inlineStr"/>
       <c r="N60" s="2" t="inlineStr"/>
       <c r="O60" s="2" t="n"/>
@@ -4980,7 +5120,7 @@
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>Tendon-pain safe entry point</t>
+          <t>Tendon-pain safe entry point; Patellar tendon / knee resilience (isometric-first)</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr"/>
@@ -5745,7 +5885,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L83" s="7" t="inlineStr"/>
+      <c r="L83" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M83" s="7" t="inlineStr"/>
       <c r="N83" s="7" t="inlineStr"/>
       <c r="O83" s="7" t="n"/>
@@ -6565,7 +6709,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N96" s="2" t="inlineStr"/>
       <c r="O96" s="2" t="n"/>
       <c r="P96" s="2" t="n"/>
@@ -6628,7 +6776,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N97" s="2" t="inlineStr"/>
       <c r="O97" s="2" t="n"/>
       <c r="P97" s="2" t="n"/>
@@ -7064,7 +7216,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M104" s="2" t="inlineStr"/>
       <c r="N104" s="2" t="inlineStr"/>
       <c r="O104" s="2" t="n"/>
@@ -7119,7 +7275,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
       <c r="M105" s="2" t="inlineStr"/>
       <c r="N105" s="2" t="inlineStr"/>
       <c r="O105" s="2" t="n"/>
@@ -7178,7 +7338,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M106" s="2" t="inlineStr"/>
       <c r="N106" s="2" t="inlineStr"/>
       <c r="O106" s="2" t="n"/>
@@ -7237,7 +7401,11 @@
           <t>Novice</t>
         </is>
       </c>
-      <c r="L107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M107" s="2" t="inlineStr"/>
       <c r="N107" s="2" t="inlineStr"/>
       <c r="O107" s="2" t="n"/>
@@ -7951,7 +8119,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N118" s="2" t="inlineStr"/>
       <c r="O118" s="2" t="n"/>
       <c r="P118" s="2" t="n"/>
@@ -8010,7 +8182,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N119" s="2" t="inlineStr"/>
       <c r="O119" s="2" t="n"/>
       <c r="P119" s="2" t="n"/>
@@ -8069,7 +8245,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N120" s="2" t="inlineStr"/>
       <c r="O120" s="2" t="n"/>
       <c r="P120" s="2" t="n"/>
@@ -8924,7 +9104,7 @@
       </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
-          <t>Off-season, Pre-season</t>
+          <t>Off-season, Pre-season, In-season</t>
         </is>
       </c>
       <c r="M134" s="2" t="inlineStr"/>
@@ -9812,7 +9992,7 @@
       </c>
       <c r="M147" s="2" t="inlineStr">
         <is>
-          <t>Supports repeated rotational throwing/diving demand (Sec. 3)</t>
+          <t>Supports repeated rotational throwing/diving demand (Sec. 3); Lower back / core resilience</t>
         </is>
       </c>
       <c r="N147" s="2" t="inlineStr"/>
@@ -10357,7 +10537,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L155" s="2" t="inlineStr"/>
+      <c r="L155" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M155" s="2" t="inlineStr"/>
       <c r="N155" s="2" t="inlineStr"/>
       <c r="O155" s="2" t="n"/>
@@ -10412,7 +10596,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L156" s="7" t="inlineStr"/>
+      <c r="L156" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M156" s="7" t="inlineStr"/>
       <c r="N156" s="7" t="inlineStr">
         <is>
@@ -10550,7 +10738,11 @@
           <t>Advanced</t>
         </is>
       </c>
-      <c r="L158" s="7" t="inlineStr"/>
+      <c r="L158" s="7" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="M158" s="7" t="inlineStr"/>
       <c r="N158" s="7" t="inlineStr"/>
       <c r="O158" s="7" t="n"/>
@@ -11425,7 +11617,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M172" s="2" t="inlineStr"/>
+      <c r="M172" s="2" t="inlineStr">
+        <is>
+          <t>Groin / adductor mobility</t>
+        </is>
+      </c>
       <c r="N172" s="2" t="inlineStr"/>
       <c r="O172" s="2" t="n"/>
       <c r="P172" s="2" t="n"/>
@@ -13024,7 +13220,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M197" s="2" t="inlineStr"/>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N197" s="2" t="inlineStr"/>
       <c r="O197" s="2" t="n"/>
       <c r="P197" s="2" t="n"/>
@@ -13087,7 +13287,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M198" s="2" t="inlineStr"/>
+      <c r="M198" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N198" s="2" t="inlineStr"/>
       <c r="O198" s="2" t="n"/>
       <c r="P198" s="2" t="n"/>
@@ -13150,7 +13354,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M199" s="2" t="inlineStr"/>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N199" s="2" t="inlineStr"/>
       <c r="O199" s="2" t="n"/>
       <c r="P199" s="2" t="n"/>
@@ -13213,7 +13421,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M200" s="2" t="inlineStr"/>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N200" s="2" t="inlineStr"/>
       <c r="O200" s="2" t="n"/>
       <c r="P200" s="2" t="n"/>
@@ -13276,7 +13488,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M201" s="2" t="inlineStr"/>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N201" s="2" t="inlineStr"/>
       <c r="O201" s="2" t="n"/>
       <c r="P201" s="2" t="n"/>
@@ -13343,7 +13559,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M202" s="2" t="inlineStr"/>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N202" s="2" t="inlineStr"/>
       <c r="O202" s="2" t="n"/>
       <c r="P202" s="2" t="n"/>
@@ -14135,7 +14355,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M214" s="7" t="inlineStr"/>
+      <c r="M214" s="7" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N214" s="7" t="inlineStr"/>
       <c r="O214" s="7" t="n"/>
       <c r="P214" s="7" t="n"/>
@@ -14675,7 +14899,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M222" s="9" t="inlineStr"/>
+      <c r="M222" s="9" t="inlineStr">
+        <is>
+          <t>Patellar tendon / knee resilience (isometric-first)</t>
+        </is>
+      </c>
       <c r="N222" s="9" t="inlineStr"/>
       <c r="O222" s="9" t="inlineStr"/>
       <c r="P222" s="9" t="n"/>
@@ -14738,7 +14966,11 @@
           <t>Off-season, Pre-season</t>
         </is>
       </c>
-      <c r="M223" s="9" t="inlineStr"/>
+      <c r="M223" s="9" t="inlineStr">
+        <is>
+          <t>Patellar tendon / knee resilience (isometric-first)</t>
+        </is>
+      </c>
       <c r="N223" s="9" t="inlineStr"/>
       <c r="O223" s="9" t="inlineStr"/>
       <c r="P223" s="9" t="n"/>
@@ -15081,7 +15313,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M228" s="9" t="inlineStr"/>
+      <c r="M228" s="9" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N228" s="9" t="inlineStr"/>
       <c r="O228" s="9" t="inlineStr"/>
       <c r="P228" s="9" t="n"/>
@@ -15152,7 +15388,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M229" s="9" t="inlineStr"/>
+      <c r="M229" s="9" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N229" s="9" t="inlineStr"/>
       <c r="O229" s="9" t="inlineStr"/>
       <c r="P229" s="9" t="n"/>
@@ -15223,7 +15463,11 @@
           <t>Off-season, Pre-season</t>
         </is>
       </c>
-      <c r="M230" s="9" t="inlineStr"/>
+      <c r="M230" s="9" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N230" s="9" t="inlineStr"/>
       <c r="O230" s="9" t="inlineStr"/>
       <c r="P230" s="9" t="n"/>
@@ -15420,7 +15664,11 @@
           <t>Off-season</t>
         </is>
       </c>
-      <c r="M233" s="9" t="inlineStr"/>
+      <c r="M233" s="9" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N233" s="9" t="inlineStr"/>
       <c r="O233" s="9" t="inlineStr"/>
       <c r="P233" s="9" t="n"/>
@@ -16118,7 +16366,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M243" s="9" t="inlineStr"/>
+      <c r="M243" s="9" t="inlineStr">
+        <is>
+          <t>Achilles tendon health (HSR)</t>
+        </is>
+      </c>
       <c r="N243" s="9" t="inlineStr"/>
       <c r="O243" s="9" t="inlineStr"/>
       <c r="P243" s="9" t="n"/>
@@ -17083,6 +17335,11 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
       <c r="Q258" t="inlineStr">
         <is>
           <t>Active</t>
@@ -19040,7 +19297,11 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M286" s="2" t="n"/>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>Lower back / core resilience</t>
+        </is>
+      </c>
       <c r="N286" s="2" t="n"/>
       <c r="O286" s="2" t="inlineStr">
         <is>
@@ -19542,7 +19803,7 @@
       </c>
       <c r="L293" s="2" t="inlineStr">
         <is>
-          <t>Pre-season</t>
+          <t>Pre-season, In-season</t>
         </is>
       </c>
       <c r="M293" s="2" t="n"/>
@@ -19834,7 +20095,7 @@
       </c>
       <c r="L297" s="2" t="inlineStr">
         <is>
-          <t>Off-season, Pre-season</t>
+          <t>Off-season, Pre-season, In-season</t>
         </is>
       </c>
       <c r="M297" s="2" t="n"/>
@@ -20218,8 +20479,1294 @@
         </is>
       </c>
     </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>UP-017</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>Incline / Elevated Push-Up</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>Upper Push</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>Easier push-up variation that builds toward the full push-up.</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G303" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H303" s="11" t="inlineStr">
+        <is>
+          <t>Hands on a bench, box or sturdy counter, body in one straight line from head to heels. Lower your chest to the edge, then push the surface away hard — the lower the surface, the harder it gets.</t>
+        </is>
+      </c>
+      <c r="I303" s="2" t="n"/>
+      <c r="J303" s="2" t="inlineStr">
+        <is>
+          <t>UP-007</t>
+        </is>
+      </c>
+      <c r="K303" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L303" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M303" s="2" t="n"/>
+      <c r="N303" s="2" t="n"/>
+      <c r="O303" s="2" t="inlineStr">
+        <is>
+          <t>Progress by lowering the hand height until you reach the floor (Push-Ups, UP-007). Typical dose: 3x8-15.</t>
+        </is>
+      </c>
+      <c r="P303" s="2" t="n"/>
+      <c r="Q303" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>UL-013</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>Band-Assisted Pull-Up / Chin-Up</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>Upper Pull</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>Builds toward unassisted pull-ups with a band taking part of your bodyweight.</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>Pull-up bar</t>
+        </is>
+      </c>
+      <c r="G304" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H304" s="11" t="inlineStr">
+        <is>
+          <t>Loop the band over the bar and under a foot or knee. Start from a full hang, pull your chest up to the bar, and lower slowly — the band helps at the bottom, so don't bounce out of it.</t>
+        </is>
+      </c>
+      <c r="I304" s="2" t="n"/>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>UL-003</t>
+        </is>
+      </c>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L304" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M304" s="2" t="n"/>
+      <c r="N304" s="2" t="n"/>
+      <c r="O304" s="2" t="inlineStr">
+        <is>
+          <t>Use a thinner band as you get stronger. Typical dose: 3x5-8. Progress to unassisted Pull-Up / Chin-Up (UL-003).</t>
+        </is>
+      </c>
+      <c r="P304" s="2" t="inlineStr">
+        <is>
+          <t>Bands</t>
+        </is>
+      </c>
+      <c r="Q304" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>UL-014</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>Band Row (Standing or Seated)</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>Upper Pull</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>Horizontal pulling with just a band, for athletes without dumbbells or cables.</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>Bands</t>
+        </is>
+      </c>
+      <c r="G305" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H305" s="11" t="inlineStr">
+        <is>
+          <t>Anchor the band at chest height, pull your elbows back and squeeze your shoulder blades together, then control the return. Don't shrug or lean back to finish the rep.</t>
+        </is>
+      </c>
+      <c r="I305" s="2" t="n"/>
+      <c r="J305" s="2" t="n"/>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L305" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M305" s="2" t="n"/>
+      <c r="N305" s="2" t="n"/>
+      <c r="O305" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x10-15. Anchor the band to a door, post or rack.</t>
+        </is>
+      </c>
+      <c r="P305" s="2" t="n"/>
+      <c r="Q305" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>SQ-007</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>Tempo Squat (Bodyweight)</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>Squat</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>Bodyweight squat with a slow lowering phase; builds control and positional strength before external load.</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H306" s="11" t="inlineStr">
+        <is>
+          <t>Take three full seconds to lower into the bottom, keep your chest up and knees tracking over your toes, then stand up with intent.</t>
+        </is>
+      </c>
+      <c r="I306" s="2" t="inlineStr">
+        <is>
+          <t>SQ-004</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>SQ-002</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L306" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M306" s="2" t="n"/>
+      <c r="N306" s="2" t="n"/>
+      <c r="O306" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x8-12 with a 3-second lowering phase.</t>
+        </is>
+      </c>
+      <c r="P306" s="2" t="n"/>
+      <c r="Q306" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>SQ-008</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>Box Squat</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>Squat</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>Barbell squat to a box, building squat strength with a consistent depth and a controlled sit-back.</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>Barbell, Rack</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H307" s="11" t="inlineStr">
+        <is>
+          <t>Sit back and down to the box with your shins vertical, pause briefly without relaxing, then drive up through the floor. Don't rock back or drop onto the box.</t>
+        </is>
+      </c>
+      <c r="I307" s="2" t="inlineStr">
+        <is>
+          <t>SQ-002</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>SQ-001</t>
+        </is>
+      </c>
+      <c r="K307" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L307" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M307" s="2" t="n"/>
+      <c r="N307" s="2" t="n"/>
+      <c r="O307" s="2" t="inlineStr">
+        <is>
+          <t>Set the box height so thighs end up about parallel. Typical dose: 3-5x3-6.</t>
+        </is>
+      </c>
+      <c r="P307" s="2" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="Q307" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>LG-008</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>Split Squat (Static)</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>Lunge / Single-Leg</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>Entry single-leg strength; a stationary split stance without the instability of a lunge.</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H308" s="11" t="inlineStr">
+        <is>
+          <t>Stand tall in a long stance, drop straight down so the back knee almost touches the floor, and drive up through the front heel. Keep your torso upright and the front knee tracking over your toes.</t>
+        </is>
+      </c>
+      <c r="I308" s="2" t="n"/>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>LG-004</t>
+        </is>
+      </c>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L308" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M308" s="2" t="n"/>
+      <c r="N308" s="2" t="n"/>
+      <c r="O308" s="2" t="inlineStr">
+        <is>
+          <t>Hold a dumbbell in each hand once it gets easy. Typical dose: 3x8-12 per leg. Replaces the retired placeholder LG-001.</t>
+        </is>
+      </c>
+      <c r="P308" s="2" t="n"/>
+      <c r="Q308" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>HG-009</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL (Bodyweight)</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>Hinge</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg hinge for balance and hamstring/glute control with no external load.</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H309" s="11" t="inlineStr">
+        <is>
+          <t>Hinge at the hip, reach long through your back leg, and keep your hips square to the floor. Stand up by squeezing the glute of the standing leg — don't let the knee lock or the back round.</t>
+        </is>
+      </c>
+      <c r="I309" s="2" t="inlineStr">
+        <is>
+          <t>HG-004</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>HG-006</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L309" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M309" s="2" t="n"/>
+      <c r="N309" s="2" t="n"/>
+      <c r="O309" s="2" t="inlineStr">
+        <is>
+          <t>Touch a wall or chair lightly for balance if needed. Typical dose: 3x6-10 per leg.</t>
+        </is>
+      </c>
+      <c r="P309" s="2" t="n"/>
+      <c r="Q309" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>HG-010</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>Good Morning (Barbell)</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>Hinge</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>Posterior-chain strength with a barbell on the back; builds hinge strength and hamstring length-under-load.</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>Barbell, Rack</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H310" s="11" t="inlineStr">
+        <is>
+          <t>Bar on your upper back, soft knees, push your hips straight back until your torso is nearly parallel to the floor, then drive the hips forward to stand. Keep your back flat the whole time.</t>
+        </is>
+      </c>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>HG-004</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>HG-005</t>
+        </is>
+      </c>
+      <c r="K310" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L310" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M310" s="2" t="n"/>
+      <c r="N310" s="2" t="n"/>
+      <c r="O310" s="2" t="inlineStr">
+        <is>
+          <t>Light weight relative to squat/deadlift. Typical dose: 3x6-10.</t>
+        </is>
+      </c>
+      <c r="P310" s="2" t="n"/>
+      <c r="Q310" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>IS-043</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>Side-Lying Hip Adduction</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Adductor</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>Adductor strengthening with no equipment; entry point to Copenhagen work.</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H311" s="11" t="inlineStr">
+        <is>
+          <t>Lie on your side with the top leg bent in front of you, lift the bottom leg straight up using the inside of the thigh, and lower slowly. Keep your hips stacked.</t>
+        </is>
+      </c>
+      <c r="I311" s="2" t="n"/>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>IS-016</t>
+        </is>
+      </c>
+      <c r="K311" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L311" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M311" s="2" t="inlineStr">
+        <is>
+          <t>Groin strain prevention</t>
+        </is>
+      </c>
+      <c r="N311" s="2" t="n"/>
+      <c r="O311" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 2-3x10-15 per side. Progress to Copenhagen Plank (IS-016, needs a bench).</t>
+        </is>
+      </c>
+      <c r="P311" s="2" t="n"/>
+      <c r="Q311" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>RS-007</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>Bodyweight Lateral Bound to Vertical Stick</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>Reflexive Strength - Loaded Movement Pattern</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>Unloaded entry to the lateral-bound reflexive chain; teaches the bound-and-stick before dumbbell load.</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H312" s="11" t="inlineStr">
+        <is>
+          <t>Bound sideways off one leg, land on the opposite leg, and stick a quiet, balanced landing before standing tall. Stop and reset if you wobble — a clean stick matters more than distance.</t>
+        </is>
+      </c>
+      <c r="I312" s="2" t="n"/>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>RS-002</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L312" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M312" s="2" t="n"/>
+      <c r="N312" s="2" t="n"/>
+      <c r="O312" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x4-6 per side. Progress to the dumbbell-loaded version (RS-002).</t>
+        </is>
+      </c>
+      <c r="P312" s="2" t="n"/>
+      <c r="Q312" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>CD-016</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>L-Drill (3-Cone)</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>Classic cone drill testing cutting, turning and acceleration through changes of direction.</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>None (cones)</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (10+ yd)</t>
+        </is>
+      </c>
+      <c r="H313" s="11" t="inlineStr">
+        <is>
+          <t>Stay low, plant hard on the outside foot, and push hard out of every turn. Round the third cone tight and keep your hips down through the whole drill.</t>
+        </is>
+      </c>
+      <c r="I313" s="2" t="n"/>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>CD-002</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L313" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M313" s="2" t="n"/>
+      <c r="N313" s="2" t="n"/>
+      <c r="O313" s="2" t="inlineStr">
+        <is>
+          <t>Cones set 5 yd apart in an L shape. Typical dose: 4-6 reps with full recovery. Time it if you want a benchmark.</t>
+        </is>
+      </c>
+      <c r="P313" s="2" t="n"/>
+      <c r="Q313" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>CD-017</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>Shuffle-to-Sprint (Self-Cued)</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>Change of Direction</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>Trains the stop-and-go from a shuffle into a sprint with no partner; the cue comes from a pre-set random sequence.</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>None (cones)</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>Requires Running Room (10+ yd)</t>
+        </is>
+      </c>
+      <c r="H314" s="11" t="inlineStr">
+        <is>
+          <t>Shuffle low and stay square, then the moment the cue hits, turn and sprint — don't wait for it, react to it. Plant hard on the first step and drive out.</t>
+        </is>
+      </c>
+      <c r="I314" s="2" t="n"/>
+      <c r="J314" s="2" t="n"/>
+      <c r="K314" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L314" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M314" s="2" t="n"/>
+      <c r="N314" s="2" t="n"/>
+      <c r="O314" s="2" t="inlineStr">
+        <is>
+          <t>Set two cones 5 yd apart and a sprint finish 10 yd away. Use a random timer or audio beep as the cue to keep it reactive without a partner. Typical dose: 4-6 reps with full recovery.</t>
+        </is>
+      </c>
+      <c r="P314" s="2" t="n"/>
+      <c r="Q314" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>PJ-039</t>
+        </is>
+      </c>
+      <c r="B315" s="2" t="inlineStr">
+        <is>
+          <t>Med-Ball Scoop Toss</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric / Jump</t>
+        </is>
+      </c>
+      <c r="E315" s="2" t="inlineStr">
+        <is>
+          <t>Triple-extension power with no barbell: ankle, knee and hip extension into a throw.</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>Medicine ball</t>
+        </is>
+      </c>
+      <c r="G315" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H315" s="11" t="inlineStr">
+        <is>
+          <t>Hinge back, swing the ball between your legs, then explode up through the hips and let the ball fly forward and up. The power comes from your legs and hips, not your arms.</t>
+        </is>
+      </c>
+      <c r="I315" s="2" t="n"/>
+      <c r="J315" s="2" t="n"/>
+      <c r="K315" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L315" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M315" s="2" t="n"/>
+      <c r="N315" s="2" t="n"/>
+      <c r="O315" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3-5x3-5, full recovery. Alternative to the Olympic lifts for athletes without a barbell.</t>
+        </is>
+      </c>
+      <c r="P315" s="2" t="n"/>
+      <c r="Q315" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>OL-009</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbell Snatch (Single-Arm)</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>Olympic Lift</t>
+        </is>
+      </c>
+      <c r="E316" s="2" t="inlineStr">
+        <is>
+          <t>Single-arm triple-extension power with a dumbbell; a lower-barrier option than the barbell snatch.</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="G316" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H316" s="11" t="inlineStr">
+        <is>
+          <t>Hinge the dumbbell back between your legs, explode through the hips, and punch the dumbbell overhead in one fluid motion. Catch it locked out with a stable shoulder.</t>
+        </is>
+      </c>
+      <c r="I316" s="2" t="inlineStr">
+        <is>
+          <t>OL-003</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="n"/>
+      <c r="K316" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L316" s="2" t="inlineStr">
+        <is>
+          <t>Off-season, Pre-season</t>
+        </is>
+      </c>
+      <c r="M316" s="2" t="n"/>
+      <c r="N316" s="2" t="n"/>
+      <c r="O316" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3-5x3-5 per arm, full recovery.</t>
+        </is>
+      </c>
+      <c r="P316" s="2" t="n"/>
+      <c r="Q316" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>IS-044</t>
+        </is>
+      </c>
+      <c r="B317" s="2" t="inlineStr">
+        <is>
+          <t>Band Biceps Curl</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Arm</t>
+        </is>
+      </c>
+      <c r="E317" s="2" t="inlineStr">
+        <is>
+          <t>Biceps work with just a band, for athletes without dumbbells or cables.</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr">
+        <is>
+          <t>Bands</t>
+        </is>
+      </c>
+      <c r="G317" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H317" s="11" t="inlineStr">
+        <is>
+          <t>Stand on the band, elbows pinned to your sides, curl up and squeeze, then lower under control. Don't swing the torso.</t>
+        </is>
+      </c>
+      <c r="I317" s="2" t="n"/>
+      <c r="J317" s="2" t="n"/>
+      <c r="K317" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L317" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M317" s="2" t="n"/>
+      <c r="N317" s="2" t="n"/>
+      <c r="O317" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x10-15.</t>
+        </is>
+      </c>
+      <c r="P317" s="2" t="n"/>
+      <c r="Q317" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>CR-035</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>Russian Twist (Bodyweight)</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>Core - Rotational Power</t>
+        </is>
+      </c>
+      <c r="E318" s="2" t="inlineStr">
+        <is>
+          <t>Entry rotational core work; trains trunk rotation without an external load.</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G318" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H318" s="11" t="inlineStr">
+        <is>
+          <t>Lean back slightly with your chest up and feet down, then rotate your whole torso side to side — don't just swing the arms. Move with control.</t>
+        </is>
+      </c>
+      <c r="I318" s="2" t="n"/>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>CR-027</t>
+        </is>
+      </c>
+      <c r="K318" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L318" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M318" s="2" t="n"/>
+      <c r="N318" s="2" t="n"/>
+      <c r="O318" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x10-20 total. Progress to Weighted Russian Twist (CR-027).</t>
+        </is>
+      </c>
+      <c r="P318" s="2" t="n"/>
+      <c r="Q318" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>IS-045</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
+        <is>
+          <t>Dead Hang / Towel Hang</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Forearm/Wrist</t>
+        </is>
+      </c>
+      <c r="E319" s="2" t="inlineStr">
+        <is>
+          <t>Grip and forearm endurance, plus shoulder decompression, with no dumbbells needed.</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>Pull-up bar</t>
+        </is>
+      </c>
+      <c r="G319" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H319" s="11" t="inlineStr">
+        <is>
+          <t>Hang from the bar with a firm grip, shoulders packed down away from your ears, and breathe. Hold as long as you can with good form.</t>
+        </is>
+      </c>
+      <c r="I319" s="2" t="n"/>
+      <c r="J319" s="2" t="n"/>
+      <c r="K319" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L319" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M319" s="2" t="n"/>
+      <c r="N319" s="2" t="n"/>
+      <c r="O319" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x20-45s. Drape a towel over the bar for a harder grip challenge.</t>
+        </is>
+      </c>
+      <c r="P319" s="2" t="n"/>
+      <c r="Q319" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>IM-027</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>Isometric Overhead Press Hold (Wall)</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>Isometric - Shoulder</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>Isometric shoulder loading for throwing resilience; builds tolerance without joint movement.</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G320" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H320" s="11" t="inlineStr">
+        <is>
+          <t>Press your forearms and hands into the wall overhead as hard as you can without shrugging your shoulders, and hold. Keep your ribs down and your neck relaxed.</t>
+        </is>
+      </c>
+      <c r="I320" s="2" t="n"/>
+      <c r="J320" s="2" t="n"/>
+      <c r="K320" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L320" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M320" s="2" t="inlineStr">
+        <is>
+          <t>Shoulder health for throwing volume</t>
+        </is>
+      </c>
+      <c r="N320" s="2" t="n"/>
+      <c r="O320" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x20-30s at moderate to hard effort.</t>
+        </is>
+      </c>
+      <c r="P320" s="2" t="n"/>
+      <c r="Q320" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q302"/>
+  <autoFilter ref="A1:Q320"/>
   <dataValidations count="6">
     <dataValidation sqref="C2:C900" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Core 50,Extended Library"</formula1>

</xml_diff>

<commit_message>
Library: add band-resisted broad jump (bilateral + single-leg) and jumping lunge
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exercise Library'!$A$1:$Q$320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exercise Library'!$A$1:$Q$323</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q320"/>
+  <dimension ref="A1:Q323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3611,7 +3611,11 @@
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr"/>
-      <c r="J47" s="7" t="inlineStr"/>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>PJ-040</t>
+        </is>
+      </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
           <t>Novice</t>
@@ -10590,7 +10594,11 @@
         </is>
       </c>
       <c r="I156" s="7" t="inlineStr"/>
-      <c r="J156" s="7" t="inlineStr"/>
+      <c r="J156" s="7" t="inlineStr">
+        <is>
+          <t>PJ-041</t>
+        </is>
+      </c>
       <c r="K156" s="7" t="inlineStr">
         <is>
           <t>Advanced</t>
@@ -21765,8 +21773,221 @@
         </is>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>PJ-040</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>Band-Resisted Broad Jump</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric / Jump</t>
+        </is>
+      </c>
+      <c r="E321" s="2" t="inlineStr">
+        <is>
+          <t>Horizontal power with band resistance; trains hard, long horizontal force through the first push and a stuck landing.</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>Bands</t>
+        </is>
+      </c>
+      <c r="G321" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly, Low-Ceiling Friendly</t>
+        </is>
+      </c>
+      <c r="H321" s="11" t="inlineStr">
+        <is>
+          <t>Anchor the band behind you at hip height. Load the hips back, swing the arms hard, and jump forward against the band's pull — then land soft with the knees bent and stick it before the band drags you back.</t>
+        </is>
+      </c>
+      <c r="I321" s="2" t="inlineStr">
+        <is>
+          <t>PJ-006</t>
+        </is>
+      </c>
+      <c r="J321" s="2" t="n"/>
+      <c r="K321" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L321" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M321" s="2" t="n"/>
+      <c r="N321" s="2" t="n"/>
+      <c r="O321" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3-4x3-4, full recovery. Use a band that lets you still reach near your normal jump distance. Use a rack, post or partner as the anchor.</t>
+        </is>
+      </c>
+      <c r="P321" s="2" t="n"/>
+      <c r="Q321" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>PJ-041</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>Band-Resisted Single-Leg Broad Hop</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric - Single-Leg / Ankle</t>
+        </is>
+      </c>
+      <c r="E322" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg horizontal power with band resistance; builds the horizontal drive and landing control that carry over to accelerating off one leg.</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr">
+        <is>
+          <t>Bands</t>
+        </is>
+      </c>
+      <c r="G322" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly, Low-Ceiling Friendly</t>
+        </is>
+      </c>
+      <c r="H322" s="11" t="inlineStr">
+        <is>
+          <t>Anchor the band behind you at hip height. Load the hips, swing the arms, and hop forward on one leg against the band — stick the landing balanced and don't let the band pull you out of position.</t>
+        </is>
+      </c>
+      <c r="I322" s="2" t="inlineStr">
+        <is>
+          <t>PJ-016</t>
+        </is>
+      </c>
+      <c r="J322" s="2" t="n"/>
+      <c r="K322" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L322" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M322" s="2" t="n"/>
+      <c r="N322" s="2" t="n"/>
+      <c r="O322" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x2-3/side, full recovery. Progress from the unresisted Single-Leg Hop for Distance (PJ-016). Bilateral version is PJ-040.</t>
+        </is>
+      </c>
+      <c r="P322" s="2" t="n"/>
+      <c r="Q322" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>PJ-042</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>Jumping Lunge (Alternating Split Jump)</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>Plyometric / Jump</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>Alternating split-stance jump that builds explosive single-leg drive, hip extension power and landing control without a barbell.</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G323" s="2" t="inlineStr">
+        <is>
+          <t>Requires Overhead Clearance</t>
+        </is>
+      </c>
+      <c r="H323" s="11" t="inlineStr">
+        <is>
+          <t>Start in a lunge, jump straight up, and switch legs in the air. Land soft in the opposite lunge with your front knee tracking over your toes, and reset your balance before the next rep.</t>
+        </is>
+      </c>
+      <c r="I323" s="2" t="inlineStr">
+        <is>
+          <t>LG-003</t>
+        </is>
+      </c>
+      <c r="J323" s="2" t="n"/>
+      <c r="K323" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L323" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M323" s="2" t="n"/>
+      <c r="N323" s="2" t="n"/>
+      <c r="O323" s="2" t="inlineStr">
+        <is>
+          <t>Typical dose: 3x6-10 total jumps (3-5 per leg), full recovery between sets. Keep quality high; stop when landings get sloppy.</t>
+        </is>
+      </c>
+      <c r="P323" s="2" t="n"/>
+      <c r="Q323" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q320"/>
+  <autoFilter ref="A1:Q323"/>
   <dataValidations count="6">
     <dataValidation sqref="C2:C900" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Core 50,Extended Library"</formula1>

</xml_diff>

<commit_message>
Conditioning: RPE-first, modality-neutral (Run/Bike/Row); add conditioning prompt rule; dedupe rest section
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -9087,7 +9087,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H134" s="11" t="inlineStr">
@@ -9115,7 +9115,7 @@
       <c r="N134" s="2" t="inlineStr"/>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>Zone 2 continuous, RPE 4-5 (talk-test: full sentences). Dose by phase — GPP/Reacclimation: 40-60 min; Hypertrophy: 30-45 min; Max Strength: 20-30 min; Power Conversion / Peak: 20-30 min as recovery only; in-season: 20-30 min optional. Run: steady jog. Bike/Row: steady cadence/split.</t>
+          <t>Work 20-60 min continuous | RPE 4-5 (talk-test: full sentences). Dose by phase — GPP/Reacclimation: 40-60 min; Hypertrophy: 30-45 min; Max Strength: 20-30 min; Power Conversion / Peak: 20-30 min as recovery only; in-season: 20-30 min optional. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P134" s="2" t="n"/>
@@ -19356,7 +19356,7 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H287" s="11" t="inlineStr">
@@ -19384,7 +19384,7 @@
       <c r="N287" s="2" t="n"/>
       <c r="O287" s="2" t="inlineStr">
         <is>
-          <t>Work 5-10s max effort | Rest 60-90s (about 1:10) | 6-10 reps, 1 block. Quality-gated: stop when output drops ~5-10%. Run: 10-30 yd sprint, walk back. Bike: assault/spin bike, seated or standing, max watts. Row: 5-8 hard strokes at max power. RPE 10.</t>
+          <t>Work 5-10s | Rest 60-90s | 6-10 reps, 1 block | RPE 10. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P287" s="2" t="n"/>
@@ -19427,7 +19427,7 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H288" s="11" t="inlineStr">
@@ -19459,7 +19459,7 @@
       <c r="N288" s="2" t="n"/>
       <c r="O288" s="2" t="inlineStr">
         <is>
-          <t>Work 10-15s max effort | Rest 90-120s (about 1:8) | 6-8 reps. Run: 40-80 yd. Bike: 10-15s all-out. Row: 10-15s, around 8-12 strokes. RPE 10.</t>
+          <t>Work 10-15s | Rest 90-120s | 6-8 reps | RPE 10. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P288" s="2" t="n"/>
@@ -19502,7 +19502,7 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H289" s="11" t="inlineStr">
@@ -19530,7 +19530,7 @@
       <c r="N289" s="2" t="n"/>
       <c r="O289" s="2" t="inlineStr">
         <is>
-          <t>Work 15-20s max effort | Rest 2-3 min (about 1:8) | 4-6 reps. Run: 100-150 yd. Bike: 15-20s all-out. Row: 15-20s, about 14-18 strokes. RPE 9-10. Advanced because the end of the interval carries real fatigue.</t>
+          <t>Work 15-20s | Rest 2-3 min | 4-6 reps | RPE 9-10. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P289" s="2" t="n"/>
@@ -19573,7 +19573,7 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H290" s="11" t="inlineStr">
@@ -19601,7 +19601,7 @@
       <c r="N290" s="2" t="n"/>
       <c r="O290" s="2" t="inlineStr">
         <is>
-          <t>Work 5-10s max | Rest 20-30s | 6-10 reps per set, 2-3 sets, 3-4 min between sets. Run: 10-20 yd sprints with a quick jog or walk back. Bike: max-watt bursts. Row: 5-8 hard strokes. RPE 9-10.</t>
+          <t>Work 5-10s | Rest 20-30s | 6-10 reps per set, 2-3 sets, 3-4 min between sets | RPE 9-10. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P290" s="2" t="n"/>
@@ -19644,7 +19644,7 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H291" s="11" t="inlineStr">
@@ -19676,7 +19676,7 @@
       <c r="N291" s="2" t="n"/>
       <c r="O291" s="2" t="inlineStr">
         <is>
-          <t>Work 10-15s | Rest 30-45s | 6-8 reps per set, 2-3 sets, 3-4 min between sets. Run: 30-60 yd sprints. Bike: hard 10-15s efforts. Row: 10-15s hard. RPE 9.</t>
+          <t>Work 10-15s | Rest 30-45s | 6-8 reps per set, 2-3 sets, 3-4 min between sets | RPE 9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P291" s="2" t="n"/>
@@ -19719,7 +19719,7 @@
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H292" s="11" t="inlineStr">
@@ -19747,7 +19747,7 @@
       <c r="N292" s="2" t="n"/>
       <c r="O292" s="2" t="inlineStr">
         <is>
-          <t>Work 30-45s as surges (e.g. 10s hard / 5s easy repeating) | Rest 45-60s | 5-7 rounds, 1-2 sets, 4-5 min between sets. Run: shuttle or straight-line surges. Bike: 10s hard / 5s easy. Row: 10s hard / 5s easy. RPE 8-9.</t>
+          <t>Work 30-45s as surges (about 10s hard / 5s easy) | Rest 45-60s | 5-7 rounds per set, 1-2 sets, 4-5 min between sets | RPE 8-9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P292" s="2" t="n"/>
@@ -19790,7 +19790,7 @@
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H293" s="11" t="inlineStr">
@@ -19818,7 +19818,7 @@
       <c r="N293" s="2" t="n"/>
       <c r="O293" s="2" t="inlineStr">
         <is>
-          <t>Work 20-30s at ~90-95% | Rest 90-150s (about 1:4-1:5) | 5-8 reps. Run: 150-200 yd. Bike: 20-30s hard. Row: 20-30s, about 18-24 strokes. RPE 8-9.</t>
+          <t>Work 20-30s | Rest 90-150s | 5-8 reps | RPE 8-9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P293" s="2" t="n"/>
@@ -19861,7 +19861,7 @@
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H294" s="11" t="inlineStr">
@@ -19893,7 +19893,7 @@
       <c r="N294" s="2" t="n"/>
       <c r="O294" s="2" t="inlineStr">
         <is>
-          <t>Work 30-45s at ~90% | Rest 90-135s (about 1:3) | 4-6 reps. Run: 200-300 yd. Bike: 30-45s hard. Row: 30-45s hard, steady rate. RPE 8-9.</t>
+          <t>Work 30-45s | Rest 90-135s | 4-6 reps | RPE 8-9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P294" s="2" t="n"/>
@@ -19936,7 +19936,7 @@
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H295" s="11" t="inlineStr">
@@ -19968,7 +19968,7 @@
       <c r="N295" s="2" t="n"/>
       <c r="O295" s="2" t="inlineStr">
         <is>
-          <t>Work 45-60s at ~90% | Rest 2-3 min (about 1:3) | 4-6 reps. Run: 300-400 yd (a 300-yd shuttle works). Bike: 45-60s hard. Row: 45-60s hard. RPE 9.</t>
+          <t>Work 45-60s | Rest 2-3 min | 4-6 reps | RPE 9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P295" s="2" t="n"/>
@@ -20011,7 +20011,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H296" s="11" t="inlineStr">
@@ -20039,7 +20039,7 @@
       <c r="N296" s="2" t="n"/>
       <c r="O296" s="2" t="inlineStr">
         <is>
-          <t>Work 60-90s at ~85-90% | Rest 3-4 min (about 1:2-1:3) | 3-5 reps. Run: 400-600 yd. Bike: 60-90s hard. Row: 60-90s hard. RPE 8-9.</t>
+          <t>Work 60-90s | Rest 3-4 min | 3-5 reps | RPE 8-9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P296" s="2" t="n"/>
@@ -20082,7 +20082,7 @@
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H297" s="11" t="inlineStr">
@@ -20110,7 +20110,7 @@
       <c r="N297" s="2" t="n"/>
       <c r="O297" s="2" t="inlineStr">
         <is>
-          <t>Work 30s at ~90-95% | Rest 30s easy | 10-20 reps (1-2 blocks of 8-10, 3 min between blocks). Run: fast, smooth running. Bike: hard, repeatable cadence. Row: 30s steady hard rate. RPE 8.</t>
+          <t>Work 30s | Rest 30s easy | 10-20 reps (1-2 blocks of 8-10, 3 min between blocks) | RPE 8. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P297" s="2" t="n"/>
@@ -20153,7 +20153,7 @@
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H298" s="11" t="inlineStr">
@@ -20185,7 +20185,7 @@
       <c r="N298" s="2" t="n"/>
       <c r="O298" s="2" t="inlineStr">
         <is>
-          <t>Work 2 min at ~90-95% HRmax | Rest 2 min easy | 5-8 reps. Run: track or road, even pace. Bike: steady hard watts. Row: steady, low-to-mid stroke rate. RPE 8.</t>
+          <t>Work 2 min | Rest 2 min easy | 5-8 reps | RPE 8. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P298" s="2" t="n"/>
@@ -20228,7 +20228,7 @@
       </c>
       <c r="G299" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H299" s="11" t="inlineStr">
@@ -20260,7 +20260,7 @@
       <c r="N299" s="2" t="n"/>
       <c r="O299" s="2" t="inlineStr">
         <is>
-          <t>Work 3 min at ~90-95% HRmax | Rest 2-3 min easy | 4-6 reps. Run: even pace. Bike: steady hard watts. Row: steady hard split. RPE 8.</t>
+          <t>Work 3 min | Rest 2-3 min easy | 4-6 reps | RPE 8. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P299" s="2" t="n"/>
@@ -20303,7 +20303,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H300" s="11" t="inlineStr">
@@ -20331,7 +20331,7 @@
       <c r="N300" s="2" t="n"/>
       <c r="O300" s="2" t="inlineStr">
         <is>
-          <t>Work 4 min at ~90-95% HRmax | Rest 3 min easy | 4 reps. Run: even pace. Bike: steady hard watts. Row: steady hard split. RPE 8-9.</t>
+          <t>Work 4 min | Rest 3 min easy | 4 reps | RPE 8-9. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P300" s="2" t="n"/>
@@ -20374,7 +20374,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H301" s="11" t="inlineStr">
@@ -20402,7 +20402,7 @@
       <c r="N301" s="2" t="n"/>
       <c r="O301" s="2" t="inlineStr">
         <is>
-          <t>Work 5-8 min at ~80-85% HRmax | Rest 1-2 min easy | 3-5 reps. Run: even pace. Bike: steady cadence. Row: steady, controlled split. RPE 6-7.</t>
+          <t>Work 5-8 min | Rest 1-2 min easy | 3-5 reps | RPE 6-7. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P301" s="2" t="n"/>
@@ -20445,7 +20445,7 @@
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>Run needs open room (see notes); Bike/Row are confined-space friendly</t>
+          <t>Confined Space Friendly (if machine-based)</t>
         </is>
       </c>
       <c r="H302" s="11" t="inlineStr">
@@ -20477,7 +20477,7 @@
       <c r="N302" s="2" t="n"/>
       <c r="O302" s="2" t="inlineStr">
         <is>
-          <t>Work 10-15 min at ~70-80% HRmax | Rest 2-3 min easy | 2-3 reps. Run: steady run. Bike: steady spin. Row: steady rhythmic rowing. RPE 5-6.</t>
+          <t>Work 10-15 min | Rest 2-3 min easy | 2-3 reps | RPE 5-6. Athlete chooses run, bike or row.</t>
         </is>
       </c>
       <c r="P302" s="2" t="n"/>

</xml_diff>

<commit_message>
Season transitions, injury chains, trap bar, equipment screen, day rename, training-age recompute, notes cleanup
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CeQY2Ci183F19sRFpY6ni2
</commit_message>
<xml_diff>
--- a/content/exercise-library/exercise-library.xlsx
+++ b/content/exercise-library/exercise-library.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q323"/>
+  <dimension ref="A1:Q332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5065,7 +5065,11 @@
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr"/>
-      <c r="O70" s="2" t="n"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>Isometric (ACTIVE knee chain end): IM-019 wall sit → IS-046 SL wall sit → IS-007 Spanish squat hold.</t>
+        </is>
+      </c>
       <c r="P70" s="2" t="n"/>
       <c r="Q70" s="2" t="inlineStr">
         <is>
@@ -5128,11 +5132,15 @@
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr"/>
-      <c r="O71" s="2" t="n"/>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>Retired — duplicate of IM-019 Isometric Wall Sit.</t>
+        </is>
+      </c>
       <c r="P71" s="2" t="n"/>
       <c r="Q71" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Retired</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5329,11 @@
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr"/>
-      <c r="O74" s="2" t="n"/>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>Calf chain: isos (active) → IS-011 single-leg calf raise (HSR step for minimal-equipment athletes) → IS-052 dumbbell version → IS-038 barbell HSR.</t>
+        </is>
+      </c>
       <c r="P74" s="2" t="n"/>
       <c r="Q74" s="2" t="inlineStr">
         <is>
@@ -14434,9 +14446,17 @@
           <t>Off-season, Pre-season</t>
         </is>
       </c>
-      <c r="M215" s="7" t="inlineStr"/>
+      <c r="M215" s="7" t="inlineStr">
+        <is>
+          <t>Patellar tendon / ACL knee resilience (HSR)</t>
+        </is>
+      </c>
       <c r="N215" s="7" t="inlineStr"/>
-      <c r="O215" s="7" t="n"/>
+      <c r="O215" s="7" t="inlineStr">
+        <is>
+          <t>Knee chain loading end point after heel-elevated squats.</t>
+        </is>
+      </c>
       <c r="P215" s="7" t="n"/>
       <c r="Q215" s="7" t="inlineStr">
         <is>
@@ -15045,9 +15065,17 @@
           <t>Year-round</t>
         </is>
       </c>
-      <c r="M224" s="9" t="inlineStr"/>
+      <c r="M224" s="9" t="inlineStr">
+        <is>
+          <t>Hamstring strain prevention</t>
+        </is>
+      </c>
       <c r="N224" s="9" t="inlineStr"/>
-      <c r="O224" s="9" t="inlineStr"/>
+      <c r="O224" s="9" t="inlineStr">
+        <is>
+          <t>Hamstring chain step 1 (ACTIVE injury): bridge iso → IS-047 walkouts.</t>
+        </is>
+      </c>
       <c r="P224" s="9" t="n"/>
       <c r="Q224" s="9" t="inlineStr">
         <is>
@@ -18011,7 +18039,7 @@
       <c r="N268" s="7" t="n"/>
       <c r="O268" s="7" t="inlineStr">
         <is>
-          <t>Technical-coordination slot on Lower Body Strength Day and Impulse Day for athletes new to training (see day-structure-templates-spec: Olympic-lift gating) — a loaded jump pattern without the Olympic lift's catch/receiving position.</t>
+          <t>Technical-coordination slot on Lower Strength Day and Lower Body Power Day for athletes new to training (see day-structure-templates-spec: Olympic-lift gating) — a loaded jump pattern without the Olympic lift's catch/receiving position.</t>
         </is>
       </c>
       <c r="P268" s="7" t="n"/>
@@ -18086,7 +18114,7 @@
       <c r="N269" s="7" t="n"/>
       <c r="O269" s="7" t="inlineStr">
         <is>
-          <t>Technical-coordination slot on Lower Body Strength Day and Impulse Day for athletes new to training (see day-structure-templates-spec: Olympic-lift gating) — bridges DB Jump up to the loads an Olympic-lift variation would use.</t>
+          <t>Technical-coordination slot on Lower Strength Day and Lower Body Power Day for athletes new to training (see day-structure-templates-spec: Olympic-lift gating) — bridges DB Jump up to the loads an Olympic-lift variation would use.</t>
         </is>
       </c>
       <c r="P269" s="7" t="n"/>
@@ -19100,7 +19128,7 @@
       <c r="N283" s="2" t="n"/>
       <c r="O283" s="2" t="inlineStr">
         <is>
-          <t>Upper-body technical-coordination slot on Upper Body Strength Day and Hypertrophy Day for athletes new to training — the beginner on-ramp into the plyo push-up progression.</t>
+          <t>Upper-body technical-coordination slot on Upper Strength 1 Day and Upper Strength 2 Day for athletes new to training — the beginner on-ramp into the plyo push-up progression.</t>
         </is>
       </c>
       <c r="P283" s="2" t="n"/>
@@ -19175,7 +19203,7 @@
       <c r="N284" s="2" t="n"/>
       <c r="O284" s="2" t="inlineStr">
         <is>
-          <t>Upper-body technical-coordination slot on Upper Body Strength Day and Hypertrophy Day for athletes new to training — bridges the kneeling regression up to the full plyo push-up.</t>
+          <t>Upper-body technical-coordination slot on Upper Strength 1 Day and Upper Strength 2 Day for athletes new to training — bridges the kneeling regression up to the full plyo push-up.</t>
         </is>
       </c>
       <c r="P284" s="2" t="n"/>
@@ -19242,7 +19270,7 @@
       <c r="N285" s="2" t="n"/>
       <c r="O285" s="2" t="inlineStr">
         <is>
-          <t>Upper-body technical-coordination slot on Upper Body Strength Day for athletes new to training — the beginner-friendly stand-in for a jerk/push-press variation until the athlete is ready for the standing, leg-driven version.</t>
+          <t>Upper-body technical-coordination slot on Upper Strength 1 Day for athletes new to training — the beginner-friendly stand-in for a jerk/push-press variation until the athlete is ready for the standing, leg-driven version.</t>
         </is>
       </c>
       <c r="P285" s="2" t="n"/>
@@ -19313,7 +19341,7 @@
       <c r="N286" s="2" t="n"/>
       <c r="O286" s="2" t="inlineStr">
         <is>
-          <t>Crunch-variation slot in Lower Body Strength Day's secondary-pattern core superset (and Upper Body Strength Day's rotational/sagittal core pairing) — the advanced-tier option alongside CR-028 (Dead Bug with Plate Pass).</t>
+          <t>Crunch-variation slot in Lower Strength Day's secondary-pattern core superset (and Upper Strength 1 Day's rotational/sagittal core pairing) — the advanced-tier option alongside CR-028 (Dead Bug with Plate Pass).</t>
         </is>
       </c>
       <c r="P286" s="2" t="n"/>
@@ -21981,6 +22009,709 @@
       </c>
       <c r="P323" s="2" t="n"/>
       <c r="Q323" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>IS-046</t>
+        </is>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>Single-Leg Wall Sit</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>Isometric - Knee/ACL</t>
+        </is>
+      </c>
+      <c r="E324" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg quad/knee isometric hold — step 2 of the knee isometric chain for active patellar/knee pain</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr">
+        <is>
+          <t>None (Bodyweight)</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H324" s="11" t="inlineStr">
+        <is>
+          <t>Back flat on the wall, one leg out in front, thigh near parallel — hold steady and breathe. Switch legs when you're done, don't rush the clock.</t>
+        </is>
+      </c>
+      <c r="I324" s="2" t="inlineStr">
+        <is>
+          <t>IM-019</t>
+        </is>
+      </c>
+      <c r="J324" s="2" t="inlineStr">
+        <is>
+          <t>IS-007</t>
+        </is>
+      </c>
+      <c r="K324" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L324" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M324" s="2" t="inlineStr">
+        <is>
+          <t>Patellar tendon / knee resilience (isometric-first)</t>
+        </is>
+      </c>
+      <c r="N324" s="2" t="n"/>
+      <c r="O324" s="2" t="inlineStr">
+        <is>
+          <t>Knee chain (ACTIVE injury): IM-019 wall sit → IS-046 single-leg wall sit → IS-007 Spanish squat. Timed hold per leg.</t>
+        </is>
+      </c>
+      <c r="P324" s="2" t="n"/>
+      <c r="Q324" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>LG-009</t>
+        </is>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>Heel-Elevated Squat (Barbell)</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>Squat</t>
+        </is>
+      </c>
+      <c r="E325" s="2" t="inlineStr">
+        <is>
+          <t>Quad-dominant squat with heels raised for greater knee travel — loading step of the knee HSR chain (patellar tendon/knee resilience)</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr">
+        <is>
+          <t>Barbell, Rack</t>
+        </is>
+      </c>
+      <c r="G325" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H325" s="11" t="inlineStr">
+        <is>
+          <t>Heels up on small plates, chest tall, and sit straight down between your hips with the knees tracking over the toes. Slow on the way down, drive the floor away.</t>
+        </is>
+      </c>
+      <c r="I325" s="2" t="inlineStr">
+        <is>
+          <t>LG-010</t>
+        </is>
+      </c>
+      <c r="J325" s="2" t="n"/>
+      <c r="K325" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L325" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M325" s="2" t="inlineStr">
+        <is>
+          <t>Patellar tendon / ACL knee resilience (HSR)</t>
+        </is>
+      </c>
+      <c r="N325" s="2" t="n"/>
+      <c r="O325" s="2" t="inlineStr">
+        <is>
+          <t>Knee chain (HISTORICAL injury / loading): heel-elevated squat (barbell or dumbbell) → pistol squat (LG-007). Use 3s down / 1-2s up tempo as HSR.</t>
+        </is>
+      </c>
+      <c r="P325" s="2" t="n"/>
+      <c r="Q325" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>LG-010</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>Heel-Elevated Squat (Dumbbell)</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>Squat</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>Quad-dominant squat with heels raised for greater knee travel — dumbbell/minimal-equipment option in the knee HSR chain</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbell</t>
+        </is>
+      </c>
+      <c r="G326" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H326" s="11" t="inlineStr">
+        <is>
+          <t>Heels up on a small plate, hold the dumbbell at your chest, and sit straight down with the knees tracking forward. Slow down, steady up.</t>
+        </is>
+      </c>
+      <c r="I326" s="2" t="inlineStr">
+        <is>
+          <t>SQ-002</t>
+        </is>
+      </c>
+      <c r="J326" s="2" t="inlineStr">
+        <is>
+          <t>LG-009</t>
+        </is>
+      </c>
+      <c r="K326" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L326" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M326" s="2" t="inlineStr">
+        <is>
+          <t>Patellar tendon / ACL knee resilience (HSR)</t>
+        </is>
+      </c>
+      <c r="N326" s="2" t="n"/>
+      <c r="O326" s="2" t="inlineStr">
+        <is>
+          <t>Knee chain (HISTORICAL injury / loading) for dumbbell-only athletes; progresses to LG-009 or LG-007.</t>
+        </is>
+      </c>
+      <c r="P326" s="2" t="n"/>
+      <c r="Q326" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>IS-047</t>
+        </is>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring Bridge Walkout</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Hamstring</t>
+        </is>
+      </c>
+      <c r="E327" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic bridge walkouts — step 2 of the hamstring chain, bridges the gap between the isometric bridge and loaded curls</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>None (Bodyweight)</t>
+        </is>
+      </c>
+      <c r="G327" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H327" s="11" t="inlineStr">
+        <is>
+          <t>Bridge up high, then walk your feet out slowly while keeping the hips up — walk back in under control, don't let the hips drop.</t>
+        </is>
+      </c>
+      <c r="I327" s="2" t="inlineStr">
+        <is>
+          <t>IM-021</t>
+        </is>
+      </c>
+      <c r="J327" s="2" t="inlineStr">
+        <is>
+          <t>IS-048</t>
+        </is>
+      </c>
+      <c r="K327" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L327" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M327" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring strain prevention</t>
+        </is>
+      </c>
+      <c r="N327" s="2" t="n"/>
+      <c r="O327" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring chain: IM-021 bridge iso → IS-047 walkouts → IS-048 SL heel-elevated bridge → IS-004/IS-049 SB curl → IS-003 Nordic.</t>
+        </is>
+      </c>
+      <c r="P327" s="2" t="n"/>
+      <c r="Q327" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>IS-048</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>Single-Leg Heel-Elevated Hamstring Bridge</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Hamstring</t>
+        </is>
+      </c>
+      <c r="E328" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg hamstring-biased bridge with the heel raised — step 3 of the hamstring chain</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr">
+        <is>
+          <t>Bench or Step</t>
+        </is>
+      </c>
+      <c r="G328" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H328" s="11" t="inlineStr">
+        <is>
+          <t>Heel up on the bench, other leg straight up in the air. Drive through the heel and bridge up high — hips level, no twisting.</t>
+        </is>
+      </c>
+      <c r="I328" s="2" t="inlineStr">
+        <is>
+          <t>IS-047</t>
+        </is>
+      </c>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>IS-004</t>
+        </is>
+      </c>
+      <c r="K328" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L328" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M328" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring strain prevention</t>
+        </is>
+      </c>
+      <c r="N328" s="2" t="n"/>
+      <c r="O328" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring chain step 3 (see IS-047).</t>
+        </is>
+      </c>
+      <c r="P328" s="2" t="n"/>
+      <c r="Q328" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>IS-049</t>
+        </is>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>Single-Leg Stability Ball Hamstring Curl</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Hamstring</t>
+        </is>
+      </c>
+      <c r="E329" s="2" t="inlineStr">
+        <is>
+          <t>Single-leg hamstring curl — progression of IS-004 on the way to the Nordic curl</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr">
+        <is>
+          <t>Stability Ball</t>
+        </is>
+      </c>
+      <c r="G329" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H329" s="11" t="inlineStr">
+        <is>
+          <t>One heel on the ball, other leg up. Bridge high and curl the ball in under you — keep the hips up the whole set.</t>
+        </is>
+      </c>
+      <c r="I329" s="2" t="inlineStr">
+        <is>
+          <t>IS-004</t>
+        </is>
+      </c>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>IS-003</t>
+        </is>
+      </c>
+      <c r="K329" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L329" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M329" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring strain prevention</t>
+        </is>
+      </c>
+      <c r="N329" s="2" t="n"/>
+      <c r="O329" s="2" t="inlineStr">
+        <is>
+          <t>Hamstring chain: bilateral IS-004 first, then this single-leg version, then IS-003 Nordic.</t>
+        </is>
+      </c>
+      <c r="P329" s="2" t="n"/>
+      <c r="Q329" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>IS-050</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>Copenhagen Dip (From Knee)</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Adductor</t>
+        </is>
+      </c>
+      <c r="E330" s="2" t="inlineStr">
+        <is>
+          <t>Dynamic adductor strengthening from a knee-supported lever — step 3 of the groin chain</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="G330" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H330" s="11" t="inlineStr">
+        <is>
+          <t>Top leg on the bench, bottom knee on the floor. Lower your hips slowly and raise back up — squeeze the inner thigh, stay long through the body.</t>
+        </is>
+      </c>
+      <c r="I330" s="2" t="inlineStr">
+        <is>
+          <t>IM-005</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr">
+        <is>
+          <t>IS-051</t>
+        </is>
+      </c>
+      <c r="K330" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L330" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M330" s="2" t="inlineStr">
+        <is>
+          <t>Groin strain prevention</t>
+        </is>
+      </c>
+      <c r="N330" s="2" t="n"/>
+      <c r="O330" s="2" t="inlineStr">
+        <is>
+          <t>Groin chain: IM-004 squeeze iso → IM-005 Copenhagen iso → IS-050 dips from knee → IS-051 dips from straight leg (IS-016 plank is an alternate).</t>
+        </is>
+      </c>
+      <c r="P330" s="2" t="n"/>
+      <c r="Q330" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>IS-051</t>
+        </is>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>Copenhagen Dip (Straight Leg)</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Adductor</t>
+        </is>
+      </c>
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>Full-lever Copenhagen dip — end of the groin chain</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H331" s="11" t="inlineStr">
+        <is>
+          <t>Top foot (or knee) on the bench, bottom leg straight off the floor. Lower your hips slowly and raise back up under control.</t>
+        </is>
+      </c>
+      <c r="I331" s="2" t="inlineStr">
+        <is>
+          <t>IS-050</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="n"/>
+      <c r="K331" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="L331" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M331" s="2" t="inlineStr">
+        <is>
+          <t>Groin strain prevention</t>
+        </is>
+      </c>
+      <c r="N331" s="2" t="n"/>
+      <c r="O331" s="2" t="inlineStr">
+        <is>
+          <t>Groin chain end point (see IS-050).</t>
+        </is>
+      </c>
+      <c r="P331" s="2" t="n"/>
+      <c r="Q331" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>IS-052</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>Single-Leg Calf Raise (Dumbbell)</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>Extended Library</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>Isolation - Calf</t>
+        </is>
+      </c>
+      <c r="E332" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbell-loaded single-leg calf raise — the HSR calf option for dumbbell-only athletes</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>Dumbbell</t>
+        </is>
+      </c>
+      <c r="G332" s="2" t="inlineStr">
+        <is>
+          <t>Confined Space Friendly</t>
+        </is>
+      </c>
+      <c r="H332" s="11" t="inlineStr">
+        <is>
+          <t>Hold a dumbbell in the same-side hand, balance on one foot, rise slowly onto the toes and lower for a 3-count. No bouncing.</t>
+        </is>
+      </c>
+      <c r="I332" s="2" t="inlineStr">
+        <is>
+          <t>IS-011</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>IS-038</t>
+        </is>
+      </c>
+      <c r="K332" s="2" t="inlineStr">
+        <is>
+          <t>Novice</t>
+        </is>
+      </c>
+      <c r="L332" s="2" t="inlineStr">
+        <is>
+          <t>Year-round</t>
+        </is>
+      </c>
+      <c r="M332" s="2" t="inlineStr">
+        <is>
+          <t>Achilles tendon health (HSR)</t>
+        </is>
+      </c>
+      <c r="N332" s="2" t="n"/>
+      <c r="O332" s="2" t="inlineStr">
+        <is>
+          <t>Calf chain: isos (active) → IS-011 single-leg calf raise (minimal equipment) → IS-052 dumbbell → IS-038 barbell HSR calf raise.</t>
+        </is>
+      </c>
+      <c r="P332" s="2" t="n"/>
+      <c r="Q332" s="2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -22176,6 +22907,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
@@ -22190,6 +22922,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
@@ -22204,6 +22937,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
@@ -22218,6 +22952,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
@@ -22232,6 +22967,7 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
@@ -22246,6 +22982,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
@@ -22260,6 +22997,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
@@ -22274,6 +23012,7 @@
         </is>
       </c>
     </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
@@ -22293,6 +23032,7 @@
         </is>
       </c>
     </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
@@ -22307,6 +23047,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
@@ -22314,6 +23055,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
@@ -22321,6 +23063,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
@@ -22328,6 +23071,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
@@ -22335,6 +23079,7 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>

</xml_diff>